<commit_message>
feat: Adjust margins of Supply and Materials DAs
</commit_message>
<xml_diff>
--- a/procurement_documents/RIS Template.xlsx
+++ b/procurement_documents/RIS Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAAD9A8F-0B9F-4359-8049-8B03BA2F9334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C5A7E5-1D22-4A10-B307-CCB47C8E6A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -192,7 +192,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="39">
+  <fonts count="38">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -379,13 +379,6 @@
     </font>
     <font>
       <sz val="16.5"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14.5"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -460,9 +453,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="1"/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -652,7 +644,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -761,32 +753,41 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="33" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="32" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -795,16 +796,202 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="23" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -814,6 +1001,9 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -826,10 +1016,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -847,168 +1034,15 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1042,65 +1076,29 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="23" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="25" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="28" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1410,11 +1408,12 @@
   <dimension ref="A1:I61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" customWidth="1"/>
-    <col min="3" max="4" width="39" customWidth="1"/>
-    <col min="5" max="8" width="8.7109375" customWidth="1"/>
-    <col min="9" max="9" width="17.42578125" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" customWidth="1"/>
+    <col min="3" max="3" width="37.28515625" customWidth="1"/>
+    <col min="4" max="4" width="35.85546875" customWidth="1"/>
+    <col min="5" max="8" width="8.42578125" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1502,14 +1501,14 @@
         <v>7</v>
       </c>
       <c r="B7" s="83"/>
-      <c r="C7" s="54" t="s">
+      <c r="C7" s="57" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="55"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="61"/>
-      <c r="G7" s="61"/>
-      <c r="H7" s="61"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9" ht="17.25">
@@ -1519,12 +1518,12 @@
       <c r="B8" s="84"/>
       <c r="C8" s="84"/>
       <c r="D8" s="85"/>
-      <c r="E8" s="56" t="s">
+      <c r="E8" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="57"/>
-      <c r="G8" s="57"/>
-      <c r="H8" s="57"/>
+      <c r="F8" s="60"/>
+      <c r="G8" s="60"/>
+      <c r="H8" s="60"/>
       <c r="I8" s="51"/>
     </row>
     <row r="9" spans="1:9" ht="21.75">
@@ -1534,10 +1533,10 @@
       <c r="B9" s="86"/>
       <c r="C9" s="86"/>
       <c r="D9" s="87"/>
-      <c r="E9" s="58" t="s">
+      <c r="E9" s="61" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="59"/>
+      <c r="F9" s="62"/>
       <c r="G9" s="88"/>
       <c r="H9" s="88"/>
       <c r="I9" s="89"/>
@@ -1566,10 +1565,10 @@
       <c r="B11" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="69" t="s">
+      <c r="C11" s="80" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="70"/>
+      <c r="D11" s="81"/>
       <c r="E11" s="42" t="s">
         <v>19</v>
       </c>
@@ -1589,8 +1588,8 @@
     <row r="12" spans="1:9" ht="13.7" customHeight="1">
       <c r="A12" s="44"/>
       <c r="B12" s="45"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="53"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="56"/>
       <c r="E12" s="48"/>
       <c r="F12" s="46"/>
       <c r="G12" s="49"/>
@@ -1600,8 +1599,8 @@
     <row r="13" spans="1:9" ht="13.7" customHeight="1">
       <c r="A13" s="44"/>
       <c r="B13" s="45"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="53"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="56"/>
       <c r="E13" s="48"/>
       <c r="F13" s="46"/>
       <c r="G13" s="49"/>
@@ -1611,8 +1610,8 @@
     <row r="14" spans="1:9" ht="13.7" customHeight="1">
       <c r="A14" s="44"/>
       <c r="B14" s="45"/>
-      <c r="C14" s="52"/>
-      <c r="D14" s="53"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="56"/>
       <c r="E14" s="48"/>
       <c r="F14" s="46"/>
       <c r="G14" s="49"/>
@@ -1622,8 +1621,8 @@
     <row r="15" spans="1:9" ht="13.7" customHeight="1">
       <c r="A15" s="44"/>
       <c r="B15" s="45"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="53"/>
+      <c r="C15" s="55"/>
+      <c r="D15" s="56"/>
       <c r="E15" s="48"/>
       <c r="F15" s="46"/>
       <c r="G15" s="49"/>
@@ -1633,8 +1632,8 @@
     <row r="16" spans="1:9" ht="13.7" customHeight="1">
       <c r="A16" s="44"/>
       <c r="B16" s="45"/>
-      <c r="C16" s="52"/>
-      <c r="D16" s="53"/>
+      <c r="C16" s="55"/>
+      <c r="D16" s="56"/>
       <c r="E16" s="48"/>
       <c r="F16" s="46"/>
       <c r="G16" s="49"/>
@@ -1644,8 +1643,8 @@
     <row r="17" spans="1:9" ht="13.7" customHeight="1">
       <c r="A17" s="44"/>
       <c r="B17" s="45"/>
-      <c r="C17" s="52"/>
-      <c r="D17" s="53"/>
+      <c r="C17" s="55"/>
+      <c r="D17" s="56"/>
       <c r="E17" s="48"/>
       <c r="F17" s="46"/>
       <c r="G17" s="49"/>
@@ -1655,8 +1654,8 @@
     <row r="18" spans="1:9" ht="13.7" customHeight="1">
       <c r="A18" s="44"/>
       <c r="B18" s="45"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="53"/>
+      <c r="C18" s="55"/>
+      <c r="D18" s="56"/>
       <c r="E18" s="48"/>
       <c r="F18" s="46"/>
       <c r="G18" s="49"/>
@@ -1666,8 +1665,8 @@
     <row r="19" spans="1:9" ht="13.7" customHeight="1">
       <c r="A19" s="44"/>
       <c r="B19" s="45"/>
-      <c r="C19" s="52"/>
-      <c r="D19" s="53"/>
+      <c r="C19" s="55"/>
+      <c r="D19" s="56"/>
       <c r="E19" s="48"/>
       <c r="F19" s="46"/>
       <c r="G19" s="49"/>
@@ -1677,8 +1676,8 @@
     <row r="20" spans="1:9" ht="13.7" customHeight="1">
       <c r="A20" s="44"/>
       <c r="B20" s="45"/>
-      <c r="C20" s="52"/>
-      <c r="D20" s="53"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="56"/>
       <c r="E20" s="48"/>
       <c r="F20" s="46"/>
       <c r="G20" s="49"/>
@@ -1688,8 +1687,8 @@
     <row r="21" spans="1:9" ht="13.7" customHeight="1">
       <c r="A21" s="44"/>
       <c r="B21" s="45"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="53"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="56"/>
       <c r="E21" s="48"/>
       <c r="F21" s="46"/>
       <c r="G21" s="49"/>
@@ -1699,8 +1698,8 @@
     <row r="22" spans="1:9" ht="13.7" customHeight="1">
       <c r="A22" s="44"/>
       <c r="B22" s="45"/>
-      <c r="C22" s="52"/>
-      <c r="D22" s="53"/>
+      <c r="C22" s="55"/>
+      <c r="D22" s="56"/>
       <c r="E22" s="48"/>
       <c r="F22" s="46"/>
       <c r="G22" s="49"/>
@@ -1710,8 +1709,8 @@
     <row r="23" spans="1:9" ht="13.7" customHeight="1">
       <c r="A23" s="44"/>
       <c r="B23" s="45"/>
-      <c r="C23" s="52"/>
-      <c r="D23" s="53"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="56"/>
       <c r="E23" s="48"/>
       <c r="F23" s="46"/>
       <c r="G23" s="49"/>
@@ -1721,8 +1720,8 @@
     <row r="24" spans="1:9" ht="13.7" customHeight="1">
       <c r="A24" s="44"/>
       <c r="B24" s="45"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="53"/>
+      <c r="C24" s="55"/>
+      <c r="D24" s="56"/>
       <c r="E24" s="48"/>
       <c r="F24" s="46"/>
       <c r="G24" s="49"/>
@@ -1732,8 +1731,8 @@
     <row r="25" spans="1:9" ht="13.7" customHeight="1">
       <c r="A25" s="44"/>
       <c r="B25" s="45"/>
-      <c r="C25" s="52"/>
-      <c r="D25" s="53"/>
+      <c r="C25" s="55"/>
+      <c r="D25" s="56"/>
       <c r="E25" s="48"/>
       <c r="F25" s="46"/>
       <c r="G25" s="49"/>
@@ -1743,8 +1742,8 @@
     <row r="26" spans="1:9" ht="13.7" customHeight="1">
       <c r="A26" s="44"/>
       <c r="B26" s="45"/>
-      <c r="C26" s="52"/>
-      <c r="D26" s="53"/>
+      <c r="C26" s="55"/>
+      <c r="D26" s="56"/>
       <c r="E26" s="48"/>
       <c r="F26" s="46"/>
       <c r="G26" s="49"/>
@@ -1754,8 +1753,8 @@
     <row r="27" spans="1:9" ht="13.7" customHeight="1">
       <c r="A27" s="44"/>
       <c r="B27" s="45"/>
-      <c r="C27" s="52"/>
-      <c r="D27" s="53"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="56"/>
       <c r="E27" s="48"/>
       <c r="F27" s="46"/>
       <c r="G27" s="49"/>
@@ -1765,8 +1764,8 @@
     <row r="28" spans="1:9" ht="13.7" customHeight="1">
       <c r="A28" s="44"/>
       <c r="B28" s="45"/>
-      <c r="C28" s="52"/>
-      <c r="D28" s="53"/>
+      <c r="C28" s="55"/>
+      <c r="D28" s="56"/>
       <c r="E28" s="48"/>
       <c r="F28" s="46"/>
       <c r="G28" s="49"/>
@@ -1776,8 +1775,8 @@
     <row r="29" spans="1:9" ht="13.7" customHeight="1">
       <c r="A29" s="44"/>
       <c r="B29" s="45"/>
-      <c r="C29" s="52"/>
-      <c r="D29" s="53"/>
+      <c r="C29" s="55"/>
+      <c r="D29" s="56"/>
       <c r="E29" s="48"/>
       <c r="F29" s="46"/>
       <c r="G29" s="49"/>
@@ -1787,8 +1786,8 @@
     <row r="30" spans="1:9" ht="13.7" customHeight="1">
       <c r="A30" s="44"/>
       <c r="B30" s="45"/>
-      <c r="C30" s="52"/>
-      <c r="D30" s="53"/>
+      <c r="C30" s="55"/>
+      <c r="D30" s="56"/>
       <c r="E30" s="48"/>
       <c r="F30" s="46"/>
       <c r="G30" s="49"/>
@@ -1798,8 +1797,8 @@
     <row r="31" spans="1:9" ht="13.7" customHeight="1">
       <c r="A31" s="44"/>
       <c r="B31" s="45"/>
-      <c r="C31" s="52"/>
-      <c r="D31" s="53"/>
+      <c r="C31" s="55"/>
+      <c r="D31" s="56"/>
       <c r="E31" s="48"/>
       <c r="F31" s="46"/>
       <c r="G31" s="49"/>
@@ -1809,8 +1808,8 @@
     <row r="32" spans="1:9" ht="13.7" customHeight="1">
       <c r="A32" s="44"/>
       <c r="B32" s="45"/>
-      <c r="C32" s="52"/>
-      <c r="D32" s="53"/>
+      <c r="C32" s="55"/>
+      <c r="D32" s="56"/>
       <c r="E32" s="48"/>
       <c r="F32" s="46"/>
       <c r="G32" s="49"/>
@@ -1820,8 +1819,8 @@
     <row r="33" spans="1:9" ht="13.7" customHeight="1">
       <c r="A33" s="44"/>
       <c r="B33" s="45"/>
-      <c r="C33" s="52"/>
-      <c r="D33" s="53"/>
+      <c r="C33" s="55"/>
+      <c r="D33" s="56"/>
       <c r="E33" s="48"/>
       <c r="F33" s="46"/>
       <c r="G33" s="49"/>
@@ -1831,8 +1830,8 @@
     <row r="34" spans="1:9" ht="13.7" customHeight="1">
       <c r="A34" s="44"/>
       <c r="B34" s="45"/>
-      <c r="C34" s="52"/>
-      <c r="D34" s="53"/>
+      <c r="C34" s="55"/>
+      <c r="D34" s="56"/>
       <c r="E34" s="48"/>
       <c r="F34" s="46"/>
       <c r="G34" s="49"/>
@@ -1842,8 +1841,8 @@
     <row r="35" spans="1:9" ht="13.7" customHeight="1">
       <c r="A35" s="44"/>
       <c r="B35" s="45"/>
-      <c r="C35" s="52"/>
-      <c r="D35" s="53"/>
+      <c r="C35" s="55"/>
+      <c r="D35" s="56"/>
       <c r="E35" s="48"/>
       <c r="F35" s="46"/>
       <c r="G35" s="49"/>
@@ -1853,8 +1852,8 @@
     <row r="36" spans="1:9" ht="13.7" customHeight="1">
       <c r="A36" s="44"/>
       <c r="B36" s="45"/>
-      <c r="C36" s="52"/>
-      <c r="D36" s="53"/>
+      <c r="C36" s="55"/>
+      <c r="D36" s="56"/>
       <c r="E36" s="48"/>
       <c r="F36" s="46"/>
       <c r="G36" s="49"/>
@@ -1864,8 +1863,8 @@
     <row r="37" spans="1:9" ht="13.7" customHeight="1">
       <c r="A37" s="44"/>
       <c r="B37" s="45"/>
-      <c r="C37" s="52"/>
-      <c r="D37" s="53"/>
+      <c r="C37" s="55"/>
+      <c r="D37" s="56"/>
       <c r="E37" s="48"/>
       <c r="F37" s="46"/>
       <c r="G37" s="49"/>
@@ -1875,8 +1874,8 @@
     <row r="38" spans="1:9" ht="13.5" customHeight="1">
       <c r="A38" s="44"/>
       <c r="B38" s="45"/>
-      <c r="C38" s="52"/>
-      <c r="D38" s="53"/>
+      <c r="C38" s="55"/>
+      <c r="D38" s="56"/>
       <c r="E38" s="48"/>
       <c r="F38" s="46"/>
       <c r="G38" s="49"/>
@@ -1886,8 +1885,8 @@
     <row r="39" spans="1:9" ht="13.7" customHeight="1">
       <c r="A39" s="44"/>
       <c r="B39" s="45"/>
-      <c r="C39" s="52"/>
-      <c r="D39" s="53"/>
+      <c r="C39" s="55"/>
+      <c r="D39" s="56"/>
       <c r="E39" s="48"/>
       <c r="F39" s="46"/>
       <c r="G39" s="49"/>
@@ -1897,8 +1896,8 @@
     <row r="40" spans="1:9" ht="13.7" customHeight="1">
       <c r="A40" s="44"/>
       <c r="B40" s="45"/>
-      <c r="C40" s="52"/>
-      <c r="D40" s="53"/>
+      <c r="C40" s="55"/>
+      <c r="D40" s="56"/>
       <c r="E40" s="48"/>
       <c r="F40" s="46"/>
       <c r="G40" s="49"/>
@@ -1908,8 +1907,8 @@
     <row r="41" spans="1:9" ht="13.7" customHeight="1">
       <c r="A41" s="44"/>
       <c r="B41" s="45"/>
-      <c r="C41" s="52"/>
-      <c r="D41" s="53"/>
+      <c r="C41" s="55"/>
+      <c r="D41" s="56"/>
       <c r="E41" s="48"/>
       <c r="F41" s="46"/>
       <c r="G41" s="49"/>
@@ -1919,8 +1918,8 @@
     <row r="42" spans="1:9" ht="13.7" customHeight="1">
       <c r="A42" s="44"/>
       <c r="B42" s="45"/>
-      <c r="C42" s="52"/>
-      <c r="D42" s="53"/>
+      <c r="C42" s="55"/>
+      <c r="D42" s="56"/>
       <c r="E42" s="48"/>
       <c r="F42" s="46"/>
       <c r="G42" s="49"/>
@@ -1930,8 +1929,8 @@
     <row r="43" spans="1:9" ht="13.7" customHeight="1">
       <c r="A43" s="44"/>
       <c r="B43" s="45"/>
-      <c r="C43" s="52"/>
-      <c r="D43" s="53"/>
+      <c r="C43" s="55"/>
+      <c r="D43" s="56"/>
       <c r="E43" s="48"/>
       <c r="F43" s="46"/>
       <c r="G43" s="49"/>
@@ -1941,8 +1940,8 @@
     <row r="44" spans="1:9" ht="13.7" customHeight="1">
       <c r="A44" s="44"/>
       <c r="B44" s="45"/>
-      <c r="C44" s="52"/>
-      <c r="D44" s="53"/>
+      <c r="C44" s="55"/>
+      <c r="D44" s="56"/>
       <c r="E44" s="48"/>
       <c r="F44" s="46"/>
       <c r="G44" s="49"/>
@@ -1952,8 +1951,8 @@
     <row r="45" spans="1:9" ht="13.7" customHeight="1">
       <c r="A45" s="44"/>
       <c r="B45" s="45"/>
-      <c r="C45" s="52"/>
-      <c r="D45" s="53"/>
+      <c r="C45" s="55"/>
+      <c r="D45" s="56"/>
       <c r="E45" s="48"/>
       <c r="F45" s="46"/>
       <c r="G45" s="49"/>
@@ -1963,8 +1962,8 @@
     <row r="46" spans="1:9" ht="13.7" customHeight="1">
       <c r="A46" s="44"/>
       <c r="B46" s="45"/>
-      <c r="C46" s="52"/>
-      <c r="D46" s="53"/>
+      <c r="C46" s="55"/>
+      <c r="D46" s="56"/>
       <c r="E46" s="48"/>
       <c r="F46" s="46"/>
       <c r="G46" s="49"/>
@@ -1974,8 +1973,8 @@
     <row r="47" spans="1:9" ht="13.7" customHeight="1">
       <c r="A47" s="44"/>
       <c r="B47" s="45"/>
-      <c r="C47" s="52"/>
-      <c r="D47" s="53"/>
+      <c r="C47" s="55"/>
+      <c r="D47" s="56"/>
       <c r="E47" s="48"/>
       <c r="F47" s="46"/>
       <c r="G47" s="49"/>
@@ -1985,8 +1984,8 @@
     <row r="48" spans="1:9" ht="13.7" customHeight="1">
       <c r="A48" s="44"/>
       <c r="B48" s="45"/>
-      <c r="C48" s="52"/>
-      <c r="D48" s="53"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="56"/>
       <c r="E48" s="48"/>
       <c r="F48" s="46"/>
       <c r="G48" s="49"/>
@@ -1996,8 +1995,8 @@
     <row r="49" spans="1:9" ht="13.7" customHeight="1">
       <c r="A49" s="44"/>
       <c r="B49" s="45"/>
-      <c r="C49" s="52"/>
-      <c r="D49" s="53"/>
+      <c r="C49" s="55"/>
+      <c r="D49" s="56"/>
       <c r="E49" s="48"/>
       <c r="F49" s="46"/>
       <c r="G49" s="49"/>
@@ -2007,8 +2006,8 @@
     <row r="50" spans="1:9" ht="13.7" hidden="1" customHeight="1">
       <c r="A50" s="44"/>
       <c r="B50" s="45"/>
-      <c r="C50" s="52"/>
-      <c r="D50" s="53"/>
+      <c r="C50" s="55"/>
+      <c r="D50" s="56"/>
       <c r="E50" s="48"/>
       <c r="F50" s="46"/>
       <c r="G50" s="49"/>
@@ -2018,8 +2017,8 @@
     <row r="51" spans="1:9" ht="13.7" customHeight="1">
       <c r="A51" s="44"/>
       <c r="B51" s="45"/>
-      <c r="C51" s="52"/>
-      <c r="D51" s="53"/>
+      <c r="C51" s="55"/>
+      <c r="D51" s="56"/>
       <c r="E51" s="48"/>
       <c r="F51" s="46"/>
       <c r="G51" s="49"/>
@@ -2029,8 +2028,8 @@
     <row r="52" spans="1:9" ht="13.7" customHeight="1">
       <c r="A52" s="44"/>
       <c r="B52" s="45"/>
-      <c r="C52" s="52"/>
-      <c r="D52" s="53"/>
+      <c r="C52" s="55"/>
+      <c r="D52" s="56"/>
       <c r="E52" s="48"/>
       <c r="F52" s="46"/>
       <c r="G52" s="49"/>
@@ -2040,8 +2039,8 @@
     <row r="53" spans="1:9" ht="13.7" customHeight="1">
       <c r="A53" s="44"/>
       <c r="B53" s="45"/>
-      <c r="C53" s="52"/>
-      <c r="D53" s="53"/>
+      <c r="C53" s="55"/>
+      <c r="D53" s="56"/>
       <c r="E53" s="48"/>
       <c r="F53" s="46"/>
       <c r="G53" s="49"/>
@@ -2051,8 +2050,8 @@
     <row r="54" spans="1:9" ht="13.7" customHeight="1">
       <c r="A54" s="44"/>
       <c r="B54" s="45"/>
-      <c r="C54" s="52"/>
-      <c r="D54" s="53"/>
+      <c r="C54" s="55"/>
+      <c r="D54" s="56"/>
       <c r="E54" s="48"/>
       <c r="F54" s="46"/>
       <c r="G54" s="49"/>
@@ -2063,96 +2062,96 @@
       <c r="A55" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="B55" s="76"/>
-      <c r="C55" s="76"/>
-      <c r="D55" s="76"/>
-      <c r="E55" s="76"/>
-      <c r="F55" s="76"/>
-      <c r="G55" s="76"/>
-      <c r="H55" s="76"/>
-      <c r="I55" s="77"/>
+      <c r="B55" s="73"/>
+      <c r="C55" s="73"/>
+      <c r="D55" s="73"/>
+      <c r="E55" s="73"/>
+      <c r="F55" s="73"/>
+      <c r="G55" s="73"/>
+      <c r="H55" s="73"/>
+      <c r="I55" s="74"/>
     </row>
     <row r="56" spans="1:9" ht="13.7" customHeight="1">
       <c r="A56" s="32"/>
-      <c r="B56" s="78"/>
-      <c r="C56" s="78"/>
-      <c r="D56" s="78"/>
-      <c r="E56" s="78"/>
-      <c r="F56" s="78"/>
-      <c r="G56" s="78"/>
-      <c r="H56" s="78"/>
-      <c r="I56" s="79"/>
+      <c r="B56" s="75"/>
+      <c r="C56" s="75"/>
+      <c r="D56" s="75"/>
+      <c r="E56" s="75"/>
+      <c r="F56" s="75"/>
+      <c r="G56" s="75"/>
+      <c r="H56" s="75"/>
+      <c r="I56" s="76"/>
     </row>
     <row r="57" spans="1:9" ht="13.7" customHeight="1">
-      <c r="A57" s="158"/>
-      <c r="B57" s="159"/>
-      <c r="C57" s="148" t="s">
+      <c r="A57" s="77"/>
+      <c r="B57" s="78"/>
+      <c r="C57" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="D57" s="148" t="s">
+      <c r="D57" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E57" s="141" t="s">
+      <c r="E57" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="F57" s="160"/>
-      <c r="G57" s="142"/>
-      <c r="H57" s="141" t="s">
+      <c r="F57" s="79"/>
+      <c r="G57" s="69"/>
+      <c r="H57" s="68" t="s">
         <v>27</v>
       </c>
-      <c r="I57" s="142"/>
+      <c r="I57" s="69"/>
     </row>
     <row r="58" spans="1:9" ht="13.7" customHeight="1">
-      <c r="A58" s="141" t="s">
+      <c r="A58" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="B58" s="142"/>
-      <c r="C58" s="151"/>
-      <c r="D58" s="151"/>
-      <c r="E58" s="154"/>
-      <c r="F58" s="155"/>
-      <c r="G58" s="156"/>
-      <c r="H58" s="154"/>
-      <c r="I58" s="156"/>
+      <c r="B58" s="69"/>
+      <c r="C58" s="54"/>
+      <c r="D58" s="54"/>
+      <c r="E58" s="70"/>
+      <c r="F58" s="71"/>
+      <c r="G58" s="72"/>
+      <c r="H58" s="70"/>
+      <c r="I58" s="72"/>
     </row>
     <row r="59" spans="1:9" ht="13.7" customHeight="1">
-      <c r="A59" s="141" t="s">
+      <c r="A59" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="B59" s="142"/>
-      <c r="C59" s="143"/>
-      <c r="D59" s="157"/>
-      <c r="E59" s="144"/>
-      <c r="F59" s="145"/>
-      <c r="G59" s="146"/>
-      <c r="H59" s="144"/>
-      <c r="I59" s="146"/>
+      <c r="B59" s="69"/>
+      <c r="C59" s="158"/>
+      <c r="D59" s="159"/>
+      <c r="E59" s="160"/>
+      <c r="F59" s="161"/>
+      <c r="G59" s="162"/>
+      <c r="H59" s="160"/>
+      <c r="I59" s="162"/>
     </row>
     <row r="60" spans="1:9" ht="13.7" customHeight="1">
-      <c r="A60" s="147" t="s">
+      <c r="A60" s="65" t="s">
         <v>30</v>
       </c>
-      <c r="B60" s="147"/>
-      <c r="C60" s="151"/>
-      <c r="D60" s="151"/>
-      <c r="E60" s="149"/>
-      <c r="F60" s="149"/>
-      <c r="G60" s="149"/>
-      <c r="H60" s="152"/>
-      <c r="I60" s="152"/>
+      <c r="B60" s="65"/>
+      <c r="C60" s="155"/>
+      <c r="D60" s="155"/>
+      <c r="E60" s="156"/>
+      <c r="F60" s="156"/>
+      <c r="G60" s="156"/>
+      <c r="H60" s="157"/>
+      <c r="I60" s="157"/>
     </row>
     <row r="61" spans="1:9" ht="13.7" customHeight="1">
-      <c r="A61" s="147" t="s">
+      <c r="A61" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="B61" s="147"/>
-      <c r="C61" s="143"/>
-      <c r="D61" s="143"/>
-      <c r="E61" s="153"/>
-      <c r="F61" s="153"/>
-      <c r="G61" s="153"/>
-      <c r="H61" s="150"/>
-      <c r="I61" s="150"/>
+      <c r="B61" s="65"/>
+      <c r="C61" s="52"/>
+      <c r="D61" s="52"/>
+      <c r="E61" s="66"/>
+      <c r="F61" s="66"/>
+      <c r="G61" s="66"/>
+      <c r="H61" s="67"/>
+      <c r="I61" s="67"/>
     </row>
   </sheetData>
   <mergeCells count="84">
@@ -2273,7 +2272,7 @@
       <c r="I1" s="113"/>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A2" s="139" t="s">
+      <c r="A2" s="153" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="115"/>
@@ -2286,13 +2285,13 @@
       <c r="I2" s="119"/>
     </row>
     <row r="3" spans="1:9" ht="17.25" customHeight="1">
-      <c r="A3" s="139" t="s">
+      <c r="A3" s="153" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="115"/>
       <c r="C3" s="115"/>
       <c r="D3" s="116"/>
-      <c r="E3" s="140" t="s">
+      <c r="E3" s="154" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="121"/>
@@ -2301,7 +2300,7 @@
       <c r="I3" s="122"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="137" t="s">
+      <c r="A4" s="151" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="96"/>
@@ -2316,7 +2315,7 @@
       <c r="I4" s="100"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="137" t="s">
+      <c r="A5" s="151" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="96"/>
@@ -2329,7 +2328,7 @@
       <c r="I5" s="100"/>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="138" t="s">
+      <c r="A6" s="152" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="103"/>
@@ -2342,7 +2341,7 @@
       <c r="I6" s="107"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="130" t="s">
+      <c r="A7" s="144" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="83"/>
@@ -2352,27 +2351,27 @@
       <c r="D7" s="126" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="60"/>
-      <c r="F7" s="61"/>
-      <c r="G7" s="61"/>
-      <c r="H7" s="61"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="131" t="s">
+      <c r="B8" s="145" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="131"/>
-      <c r="D8" s="132"/>
-      <c r="E8" s="60" t="s">
+      <c r="C8" s="145"/>
+      <c r="D8" s="146"/>
+      <c r="E8" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
+      <c r="F8" s="64"/>
+      <c r="G8" s="64"/>
+      <c r="H8" s="64"/>
       <c r="I8" s="3" t="s">
         <v>34</v>
       </c>
@@ -2381,34 +2380,34 @@
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="131" t="s">
+      <c r="B9" s="145" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="131"/>
-      <c r="D9" s="132"/>
-      <c r="E9" s="60" t="s">
+      <c r="C9" s="145"/>
+      <c r="D9" s="146"/>
+      <c r="E9" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="61"/>
-      <c r="G9" s="133" t="s">
+      <c r="F9" s="64"/>
+      <c r="G9" s="147" t="s">
         <v>36</v>
       </c>
-      <c r="H9" s="133"/>
-      <c r="I9" s="134"/>
+      <c r="H9" s="147"/>
+      <c r="I9" s="148"/>
     </row>
     <row r="10" spans="1:9" ht="15" customHeight="1">
-      <c r="A10" s="135" t="s">
+      <c r="A10" s="149" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="91"/>
       <c r="C10" s="91"/>
       <c r="D10" s="91"/>
       <c r="E10" s="92"/>
-      <c r="F10" s="136" t="s">
+      <c r="F10" s="150" t="s">
         <v>14</v>
       </c>
       <c r="G10" s="94"/>
-      <c r="H10" s="135" t="s">
+      <c r="H10" s="149" t="s">
         <v>15</v>
       </c>
       <c r="I10" s="92"/>
@@ -2420,10 +2419,10 @@
       <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="127" t="s">
+      <c r="C11" s="135" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="70"/>
+      <c r="D11" s="81"/>
       <c r="E11" s="5" t="s">
         <v>19</v>
       </c>
@@ -2939,111 +2938,111 @@
       <c r="A55" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="B55" s="128" t="s">
+      <c r="B55" s="141" t="s">
         <v>45</v>
       </c>
-      <c r="C55" s="128"/>
-      <c r="D55" s="128"/>
-      <c r="E55" s="128"/>
-      <c r="F55" s="128"/>
-      <c r="G55" s="128"/>
-      <c r="H55" s="128"/>
-      <c r="I55" s="129"/>
+      <c r="C55" s="141"/>
+      <c r="D55" s="141"/>
+      <c r="E55" s="141"/>
+      <c r="F55" s="141"/>
+      <c r="G55" s="141"/>
+      <c r="H55" s="141"/>
+      <c r="I55" s="142"/>
     </row>
     <row r="56" spans="1:13" ht="13.7" customHeight="1">
       <c r="A56" s="32"/>
-      <c r="B56" s="78"/>
-      <c r="C56" s="78"/>
-      <c r="D56" s="78"/>
-      <c r="E56" s="78"/>
-      <c r="F56" s="78"/>
-      <c r="G56" s="78"/>
-      <c r="H56" s="78"/>
-      <c r="I56" s="79"/>
+      <c r="B56" s="75"/>
+      <c r="C56" s="75"/>
+      <c r="D56" s="75"/>
+      <c r="E56" s="75"/>
+      <c r="F56" s="75"/>
+      <c r="G56" s="75"/>
+      <c r="H56" s="75"/>
+      <c r="I56" s="76"/>
     </row>
     <row r="57" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A57" s="80"/>
-      <c r="B57" s="65"/>
+      <c r="A57" s="130"/>
+      <c r="B57" s="131"/>
       <c r="C57" s="33" t="s">
         <v>24</v>
       </c>
       <c r="D57" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="E57" s="80" t="s">
+      <c r="E57" s="130" t="s">
         <v>26</v>
       </c>
-      <c r="F57" s="81"/>
-      <c r="G57" s="65"/>
-      <c r="H57" s="80" t="s">
+      <c r="F57" s="143"/>
+      <c r="G57" s="131"/>
+      <c r="H57" s="130" t="s">
         <v>27</v>
       </c>
-      <c r="I57" s="65"/>
+      <c r="I57" s="131"/>
     </row>
     <row r="58" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A58" s="80" t="s">
+      <c r="A58" s="130" t="s">
         <v>28</v>
       </c>
-      <c r="B58" s="65"/>
+      <c r="B58" s="131"/>
       <c r="C58" s="34"/>
       <c r="D58" s="34"/>
-      <c r="E58" s="66"/>
-      <c r="F58" s="67"/>
-      <c r="G58" s="68"/>
-      <c r="H58" s="66"/>
-      <c r="I58" s="68"/>
+      <c r="E58" s="132"/>
+      <c r="F58" s="133"/>
+      <c r="G58" s="134"/>
+      <c r="H58" s="132"/>
+      <c r="I58" s="134"/>
     </row>
     <row r="59" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A59" s="127" t="s">
+      <c r="A59" s="135" t="s">
         <v>29</v>
       </c>
-      <c r="B59" s="70"/>
+      <c r="B59" s="81"/>
       <c r="C59" s="35" t="s">
         <v>51</v>
       </c>
       <c r="D59" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="E59" s="71" t="s">
+      <c r="E59" s="136" t="s">
         <v>49</v>
       </c>
-      <c r="F59" s="72"/>
-      <c r="G59" s="73"/>
-      <c r="H59" s="74" t="s">
+      <c r="F59" s="137"/>
+      <c r="G59" s="138"/>
+      <c r="H59" s="139" t="s">
         <v>46</v>
       </c>
-      <c r="I59" s="75"/>
+      <c r="I59" s="140"/>
     </row>
     <row r="60" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A60" s="62" t="s">
+      <c r="A60" s="127" t="s">
         <v>30</v>
       </c>
-      <c r="B60" s="62"/>
+      <c r="B60" s="127"/>
       <c r="C60" s="36"/>
       <c r="D60" s="37"/>
-      <c r="E60" s="63"/>
-      <c r="F60" s="63"/>
-      <c r="G60" s="63"/>
-      <c r="H60" s="64" t="s">
+      <c r="E60" s="128"/>
+      <c r="F60" s="128"/>
+      <c r="G60" s="128"/>
+      <c r="H60" s="129" t="s">
         <v>47</v>
       </c>
-      <c r="I60" s="64"/>
+      <c r="I60" s="129"/>
       <c r="M60" s="38"/>
     </row>
     <row r="61" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A61" s="62" t="s">
+      <c r="A61" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="B61" s="62"/>
+      <c r="B61" s="127"/>
       <c r="C61" s="36"/>
       <c r="D61" s="37"/>
-      <c r="E61" s="63"/>
-      <c r="F61" s="63"/>
-      <c r="G61" s="63"/>
-      <c r="H61" s="64" t="s">
+      <c r="E61" s="128"/>
+      <c r="F61" s="128"/>
+      <c r="G61" s="128"/>
+      <c r="H61" s="129" t="s">
         <v>48</v>
       </c>
-      <c r="I61" s="64"/>
+      <c r="I61" s="129"/>
     </row>
     <row r="62" spans="1:13" ht="13.7" customHeight="1">
       <c r="M62" s="39"/>

</xml_diff>

<commit_message>
feat: generate MR QR code for RIS
</commit_message>
<xml_diff>
--- a/procurement_documents/RIS Template.xlsx
+++ b/procurement_documents/RIS Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C5A7E5-1D22-4A10-B307-CCB47C8E6A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0397C4BD-12CE-4064-8D03-40495EDBF07F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="54">
   <si>
     <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES</t>
   </si>
@@ -183,6 +183,12 @@
   </si>
   <si>
     <t>Created PR</t>
+  </si>
+  <si>
+    <t>mr_qr_code</t>
+  </si>
+  <si>
+    <t>Scan to receive item/s</t>
   </si>
 </sst>
 </file>
@@ -192,7 +198,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="41">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -455,6 +461,30 @@
     <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -644,7 +674,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="163">
+  <cellXfs count="173">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -784,11 +814,206 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="28" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="23" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -806,179 +1031,38 @@
     <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="23" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -986,11 +1070,47 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1001,104 +1121,44 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="28" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1405,170 +1465,170 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" customWidth="1"/>
-    <col min="3" max="3" width="37.28515625" customWidth="1"/>
-    <col min="4" max="4" width="35.85546875" customWidth="1"/>
-    <col min="5" max="8" width="8.42578125" customWidth="1"/>
-    <col min="9" max="9" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="41" customWidth="1"/>
+    <col min="4" max="4" width="39.42578125" customWidth="1"/>
+    <col min="5" max="8" width="9.140625" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="108"/>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="110"/>
-      <c r="E1" s="111"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="113"/>
+    <row r="1" spans="1:9" ht="15" customHeight="1">
+      <c r="A1" s="58"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="164"/>
+      <c r="F1" s="165"/>
+      <c r="G1" s="165"/>
+      <c r="H1" s="165"/>
+      <c r="I1" s="166"/>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A2" s="114" t="s">
+      <c r="A2" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="115"/>
-      <c r="C2" s="115"/>
-      <c r="D2" s="116"/>
-      <c r="E2" s="117"/>
-      <c r="F2" s="118"/>
-      <c r="G2" s="118"/>
-      <c r="H2" s="118"/>
-      <c r="I2" s="119"/>
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="167"/>
+      <c r="F2" s="168"/>
+      <c r="G2" s="168"/>
+      <c r="H2" s="168"/>
+      <c r="I2" s="169"/>
     </row>
     <row r="3" spans="1:9" ht="17.25" customHeight="1">
-      <c r="A3" s="114" t="s">
+      <c r="A3" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="115"/>
-      <c r="C3" s="115"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="120" t="s">
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="121"/>
-      <c r="G3" s="121"/>
-      <c r="H3" s="121"/>
-      <c r="I3" s="122"/>
-    </row>
-    <row r="4" spans="1:9" ht="19.5">
-      <c r="A4" s="95" t="s">
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="72"/>
+    </row>
+    <row r="4" spans="1:9" ht="15" customHeight="1">
+      <c r="A4" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="96"/>
-      <c r="C4" s="96"/>
-      <c r="D4" s="97"/>
-      <c r="E4" s="98" t="s">
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="75"/>
+      <c r="E4" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="99"/>
-      <c r="G4" s="99"/>
-      <c r="H4" s="99"/>
-      <c r="I4" s="100"/>
-    </row>
-    <row r="5" spans="1:9" ht="19.5">
-      <c r="A5" s="95" t="s">
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
+      <c r="I4" s="78"/>
+    </row>
+    <row r="5" spans="1:9" ht="15" customHeight="1">
+      <c r="A5" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="96"/>
-      <c r="C5" s="96"/>
-      <c r="D5" s="97"/>
-      <c r="E5" s="101"/>
-      <c r="F5" s="99"/>
-      <c r="G5" s="99"/>
-      <c r="H5" s="99"/>
-      <c r="I5" s="100"/>
-    </row>
-    <row r="6" spans="1:9" ht="19.5">
-      <c r="A6" s="102" t="s">
+      <c r="B5" s="74"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="75"/>
+      <c r="E5" s="79"/>
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="77"/>
+      <c r="I5" s="78"/>
+    </row>
+    <row r="6" spans="1:9" ht="15" customHeight="1">
+      <c r="A6" s="80" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="103"/>
-      <c r="C6" s="103"/>
-      <c r="D6" s="104"/>
-      <c r="E6" s="105"/>
-      <c r="F6" s="106"/>
-      <c r="G6" s="106"/>
-      <c r="H6" s="106"/>
-      <c r="I6" s="107"/>
-    </row>
-    <row r="7" spans="1:9" ht="21.75">
-      <c r="A7" s="82" t="s">
+      <c r="B6" s="81"/>
+      <c r="C6" s="81"/>
+      <c r="D6" s="82"/>
+      <c r="E6" s="83"/>
+      <c r="F6" s="84"/>
+      <c r="G6" s="84"/>
+      <c r="H6" s="84"/>
+      <c r="I6" s="85"/>
+    </row>
+    <row r="7" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A7" s="162" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="57" t="s">
+      <c r="B7" s="163"/>
+      <c r="C7" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="58"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64"/>
-      <c r="H7" s="64"/>
+      <c r="D7" s="123"/>
+      <c r="E7" s="128"/>
+      <c r="F7" s="129"/>
+      <c r="G7" s="129"/>
+      <c r="H7" s="129"/>
       <c r="I7" s="1"/>
     </row>
-    <row r="8" spans="1:9" ht="17.25">
+    <row r="8" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="84"/>
-      <c r="C8" s="84"/>
-      <c r="D8" s="85"/>
-      <c r="E8" s="59" t="s">
+      <c r="B8" s="87"/>
+      <c r="C8" s="87"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="124" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="60"/>
-      <c r="G8" s="60"/>
-      <c r="H8" s="60"/>
+      <c r="F8" s="125"/>
+      <c r="G8" s="125"/>
+      <c r="H8" s="125"/>
       <c r="I8" s="51"/>
     </row>
-    <row r="9" spans="1:9" ht="21.75">
+    <row r="9" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A9" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="86"/>
-      <c r="C9" s="86"/>
-      <c r="D9" s="87"/>
-      <c r="E9" s="61" t="s">
+      <c r="B9" s="89"/>
+      <c r="C9" s="89"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="126" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="62"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="89"/>
-    </row>
-    <row r="10" spans="1:9" ht="15" customHeight="1">
-      <c r="A10" s="90" t="s">
+      <c r="F9" s="127"/>
+      <c r="G9" s="91"/>
+      <c r="H9" s="91"/>
+      <c r="I9" s="92"/>
+    </row>
+    <row r="10" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A10" s="93" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="91"/>
-      <c r="C10" s="91"/>
-      <c r="D10" s="91"/>
-      <c r="E10" s="92"/>
-      <c r="F10" s="93" t="s">
+      <c r="B10" s="94"/>
+      <c r="C10" s="94"/>
+      <c r="D10" s="94"/>
+      <c r="E10" s="95"/>
+      <c r="F10" s="96" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="94"/>
-      <c r="H10" s="90" t="s">
+      <c r="G10" s="97"/>
+      <c r="H10" s="93" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="92"/>
-    </row>
-    <row r="11" spans="1:9" ht="43.5">
+      <c r="I10" s="95"/>
+    </row>
+    <row r="11" spans="1:9" ht="45" customHeight="1">
       <c r="A11" s="41" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="80" t="s">
+      <c r="C11" s="100" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="81"/>
+      <c r="D11" s="101"/>
       <c r="E11" s="42" t="s">
         <v>19</v>
       </c>
@@ -1585,610 +1645,620 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="13.7" customHeight="1">
+    <row r="12" spans="1:9" ht="15" customHeight="1">
       <c r="A12" s="44"/>
       <c r="B12" s="45"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="56"/>
+      <c r="C12" s="98"/>
+      <c r="D12" s="99"/>
       <c r="E12" s="48"/>
       <c r="F12" s="46"/>
       <c r="G12" s="49"/>
       <c r="H12" s="45"/>
       <c r="I12" s="50"/>
     </row>
-    <row r="13" spans="1:9" ht="13.7" customHeight="1">
+    <row r="13" spans="1:9" ht="15" customHeight="1">
       <c r="A13" s="44"/>
       <c r="B13" s="45"/>
-      <c r="C13" s="55"/>
-      <c r="D13" s="56"/>
+      <c r="C13" s="98"/>
+      <c r="D13" s="99"/>
       <c r="E13" s="48"/>
       <c r="F13" s="46"/>
       <c r="G13" s="49"/>
       <c r="H13" s="45"/>
       <c r="I13" s="50"/>
     </row>
-    <row r="14" spans="1:9" ht="13.7" customHeight="1">
+    <row r="14" spans="1:9" ht="15" customHeight="1">
       <c r="A14" s="44"/>
       <c r="B14" s="45"/>
-      <c r="C14" s="55"/>
-      <c r="D14" s="56"/>
+      <c r="C14" s="98"/>
+      <c r="D14" s="99"/>
       <c r="E14" s="48"/>
       <c r="F14" s="46"/>
       <c r="G14" s="49"/>
       <c r="H14" s="45"/>
       <c r="I14" s="50"/>
     </row>
-    <row r="15" spans="1:9" ht="13.7" customHeight="1">
+    <row r="15" spans="1:9" ht="15" customHeight="1">
       <c r="A15" s="44"/>
       <c r="B15" s="45"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="56"/>
+      <c r="C15" s="98"/>
+      <c r="D15" s="99"/>
       <c r="E15" s="48"/>
       <c r="F15" s="46"/>
       <c r="G15" s="49"/>
       <c r="H15" s="45"/>
       <c r="I15" s="50"/>
     </row>
-    <row r="16" spans="1:9" ht="13.7" customHeight="1">
+    <row r="16" spans="1:9" ht="15" customHeight="1">
       <c r="A16" s="44"/>
       <c r="B16" s="45"/>
-      <c r="C16" s="55"/>
-      <c r="D16" s="56"/>
+      <c r="C16" s="98"/>
+      <c r="D16" s="99"/>
       <c r="E16" s="48"/>
       <c r="F16" s="46"/>
       <c r="G16" s="49"/>
       <c r="H16" s="45"/>
       <c r="I16" s="50"/>
     </row>
-    <row r="17" spans="1:9" ht="13.7" customHeight="1">
+    <row r="17" spans="1:9" ht="15" customHeight="1">
       <c r="A17" s="44"/>
       <c r="B17" s="45"/>
-      <c r="C17" s="55"/>
-      <c r="D17" s="56"/>
+      <c r="C17" s="98"/>
+      <c r="D17" s="99"/>
       <c r="E17" s="48"/>
       <c r="F17" s="46"/>
       <c r="G17" s="49"/>
       <c r="H17" s="45"/>
       <c r="I17" s="50"/>
     </row>
-    <row r="18" spans="1:9" ht="13.7" customHeight="1">
+    <row r="18" spans="1:9" ht="15" customHeight="1">
       <c r="A18" s="44"/>
       <c r="B18" s="45"/>
-      <c r="C18" s="55"/>
-      <c r="D18" s="56"/>
+      <c r="C18" s="98"/>
+      <c r="D18" s="99"/>
       <c r="E18" s="48"/>
       <c r="F18" s="46"/>
       <c r="G18" s="49"/>
       <c r="H18" s="45"/>
       <c r="I18" s="50"/>
     </row>
-    <row r="19" spans="1:9" ht="13.7" customHeight="1">
+    <row r="19" spans="1:9" ht="15" customHeight="1">
       <c r="A19" s="44"/>
       <c r="B19" s="45"/>
-      <c r="C19" s="55"/>
-      <c r="D19" s="56"/>
+      <c r="C19" s="98"/>
+      <c r="D19" s="99"/>
       <c r="E19" s="48"/>
       <c r="F19" s="46"/>
       <c r="G19" s="49"/>
       <c r="H19" s="45"/>
       <c r="I19" s="50"/>
     </row>
-    <row r="20" spans="1:9" ht="13.7" customHeight="1">
+    <row r="20" spans="1:9" ht="15" customHeight="1">
       <c r="A20" s="44"/>
       <c r="B20" s="45"/>
-      <c r="C20" s="55"/>
-      <c r="D20" s="56"/>
+      <c r="C20" s="98"/>
+      <c r="D20" s="99"/>
       <c r="E20" s="48"/>
       <c r="F20" s="46"/>
       <c r="G20" s="49"/>
       <c r="H20" s="45"/>
       <c r="I20" s="50"/>
     </row>
-    <row r="21" spans="1:9" ht="13.7" customHeight="1">
+    <row r="21" spans="1:9" ht="15" customHeight="1">
       <c r="A21" s="44"/>
       <c r="B21" s="45"/>
-      <c r="C21" s="55"/>
-      <c r="D21" s="56"/>
+      <c r="C21" s="98"/>
+      <c r="D21" s="99"/>
       <c r="E21" s="48"/>
       <c r="F21" s="46"/>
       <c r="G21" s="49"/>
       <c r="H21" s="45"/>
       <c r="I21" s="50"/>
     </row>
-    <row r="22" spans="1:9" ht="13.7" customHeight="1">
+    <row r="22" spans="1:9" ht="15" customHeight="1">
       <c r="A22" s="44"/>
       <c r="B22" s="45"/>
-      <c r="C22" s="55"/>
-      <c r="D22" s="56"/>
+      <c r="C22" s="98"/>
+      <c r="D22" s="99"/>
       <c r="E22" s="48"/>
       <c r="F22" s="46"/>
       <c r="G22" s="49"/>
       <c r="H22" s="45"/>
       <c r="I22" s="50"/>
     </row>
-    <row r="23" spans="1:9" ht="13.7" customHeight="1">
+    <row r="23" spans="1:9" ht="15" customHeight="1">
       <c r="A23" s="44"/>
       <c r="B23" s="45"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="56"/>
+      <c r="C23" s="98"/>
+      <c r="D23" s="99"/>
       <c r="E23" s="48"/>
       <c r="F23" s="46"/>
       <c r="G23" s="49"/>
       <c r="H23" s="45"/>
       <c r="I23" s="50"/>
     </row>
-    <row r="24" spans="1:9" ht="13.7" customHeight="1">
+    <row r="24" spans="1:9" ht="15" customHeight="1">
       <c r="A24" s="44"/>
       <c r="B24" s="45"/>
-      <c r="C24" s="55"/>
-      <c r="D24" s="56"/>
+      <c r="C24" s="98"/>
+      <c r="D24" s="99"/>
       <c r="E24" s="48"/>
       <c r="F24" s="46"/>
       <c r="G24" s="49"/>
       <c r="H24" s="45"/>
       <c r="I24" s="50"/>
     </row>
-    <row r="25" spans="1:9" ht="13.7" customHeight="1">
+    <row r="25" spans="1:9" ht="15" customHeight="1">
       <c r="A25" s="44"/>
       <c r="B25" s="45"/>
-      <c r="C25" s="55"/>
-      <c r="D25" s="56"/>
+      <c r="C25" s="98"/>
+      <c r="D25" s="99"/>
       <c r="E25" s="48"/>
       <c r="F25" s="46"/>
       <c r="G25" s="49"/>
       <c r="H25" s="45"/>
       <c r="I25" s="50"/>
     </row>
-    <row r="26" spans="1:9" ht="13.7" customHeight="1">
+    <row r="26" spans="1:9" ht="15" customHeight="1">
       <c r="A26" s="44"/>
       <c r="B26" s="45"/>
-      <c r="C26" s="55"/>
-      <c r="D26" s="56"/>
+      <c r="C26" s="98"/>
+      <c r="D26" s="99"/>
       <c r="E26" s="48"/>
       <c r="F26" s="46"/>
       <c r="G26" s="49"/>
       <c r="H26" s="45"/>
       <c r="I26" s="50"/>
     </row>
-    <row r="27" spans="1:9" ht="13.7" customHeight="1">
+    <row r="27" spans="1:9" ht="15" customHeight="1">
       <c r="A27" s="44"/>
       <c r="B27" s="45"/>
-      <c r="C27" s="55"/>
-      <c r="D27" s="56"/>
+      <c r="C27" s="98"/>
+      <c r="D27" s="99"/>
       <c r="E27" s="48"/>
       <c r="F27" s="46"/>
       <c r="G27" s="49"/>
       <c r="H27" s="45"/>
       <c r="I27" s="50"/>
     </row>
-    <row r="28" spans="1:9" ht="13.7" customHeight="1">
+    <row r="28" spans="1:9" ht="15" customHeight="1">
       <c r="A28" s="44"/>
       <c r="B28" s="45"/>
-      <c r="C28" s="55"/>
-      <c r="D28" s="56"/>
+      <c r="C28" s="98"/>
+      <c r="D28" s="99"/>
       <c r="E28" s="48"/>
       <c r="F28" s="46"/>
       <c r="G28" s="49"/>
       <c r="H28" s="45"/>
       <c r="I28" s="50"/>
     </row>
-    <row r="29" spans="1:9" ht="13.7" customHeight="1">
+    <row r="29" spans="1:9" ht="15" customHeight="1">
       <c r="A29" s="44"/>
       <c r="B29" s="45"/>
-      <c r="C29" s="55"/>
-      <c r="D29" s="56"/>
+      <c r="C29" s="98"/>
+      <c r="D29" s="99"/>
       <c r="E29" s="48"/>
       <c r="F29" s="46"/>
       <c r="G29" s="49"/>
       <c r="H29" s="45"/>
       <c r="I29" s="50"/>
     </row>
-    <row r="30" spans="1:9" ht="13.7" customHeight="1">
+    <row r="30" spans="1:9" ht="15" customHeight="1">
       <c r="A30" s="44"/>
       <c r="B30" s="45"/>
-      <c r="C30" s="55"/>
-      <c r="D30" s="56"/>
+      <c r="C30" s="98"/>
+      <c r="D30" s="99"/>
       <c r="E30" s="48"/>
       <c r="F30" s="46"/>
       <c r="G30" s="49"/>
       <c r="H30" s="45"/>
       <c r="I30" s="50"/>
     </row>
-    <row r="31" spans="1:9" ht="13.7" customHeight="1">
+    <row r="31" spans="1:9" ht="15" customHeight="1">
       <c r="A31" s="44"/>
       <c r="B31" s="45"/>
-      <c r="C31" s="55"/>
-      <c r="D31" s="56"/>
+      <c r="C31" s="98"/>
+      <c r="D31" s="99"/>
       <c r="E31" s="48"/>
       <c r="F31" s="46"/>
       <c r="G31" s="49"/>
       <c r="H31" s="45"/>
       <c r="I31" s="50"/>
     </row>
-    <row r="32" spans="1:9" ht="13.7" customHeight="1">
+    <row r="32" spans="1:9" ht="15" customHeight="1">
       <c r="A32" s="44"/>
       <c r="B32" s="45"/>
-      <c r="C32" s="55"/>
-      <c r="D32" s="56"/>
+      <c r="C32" s="98"/>
+      <c r="D32" s="99"/>
       <c r="E32" s="48"/>
       <c r="F32" s="46"/>
       <c r="G32" s="49"/>
       <c r="H32" s="45"/>
       <c r="I32" s="50"/>
     </row>
-    <row r="33" spans="1:9" ht="13.7" customHeight="1">
+    <row r="33" spans="1:9" ht="15" customHeight="1">
       <c r="A33" s="44"/>
       <c r="B33" s="45"/>
-      <c r="C33" s="55"/>
-      <c r="D33" s="56"/>
+      <c r="C33" s="98"/>
+      <c r="D33" s="99"/>
       <c r="E33" s="48"/>
       <c r="F33" s="46"/>
       <c r="G33" s="49"/>
       <c r="H33" s="45"/>
       <c r="I33" s="50"/>
     </row>
-    <row r="34" spans="1:9" ht="13.7" customHeight="1">
+    <row r="34" spans="1:9" ht="15" customHeight="1">
       <c r="A34" s="44"/>
       <c r="B34" s="45"/>
-      <c r="C34" s="55"/>
-      <c r="D34" s="56"/>
+      <c r="C34" s="98"/>
+      <c r="D34" s="99"/>
       <c r="E34" s="48"/>
       <c r="F34" s="46"/>
       <c r="G34" s="49"/>
       <c r="H34" s="45"/>
       <c r="I34" s="50"/>
     </row>
-    <row r="35" spans="1:9" ht="13.7" customHeight="1">
+    <row r="35" spans="1:9" ht="15" customHeight="1">
       <c r="A35" s="44"/>
       <c r="B35" s="45"/>
-      <c r="C35" s="55"/>
-      <c r="D35" s="56"/>
+      <c r="C35" s="98"/>
+      <c r="D35" s="99"/>
       <c r="E35" s="48"/>
       <c r="F35" s="46"/>
       <c r="G35" s="49"/>
       <c r="H35" s="45"/>
       <c r="I35" s="50"/>
     </row>
-    <row r="36" spans="1:9" ht="13.7" customHeight="1">
+    <row r="36" spans="1:9" ht="15" customHeight="1">
       <c r="A36" s="44"/>
       <c r="B36" s="45"/>
-      <c r="C36" s="55"/>
-      <c r="D36" s="56"/>
+      <c r="C36" s="98"/>
+      <c r="D36" s="99"/>
       <c r="E36" s="48"/>
       <c r="F36" s="46"/>
       <c r="G36" s="49"/>
       <c r="H36" s="45"/>
       <c r="I36" s="50"/>
     </row>
-    <row r="37" spans="1:9" ht="13.7" customHeight="1">
+    <row r="37" spans="1:9" ht="15" customHeight="1">
       <c r="A37" s="44"/>
       <c r="B37" s="45"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="56"/>
+      <c r="C37" s="98"/>
+      <c r="D37" s="99"/>
       <c r="E37" s="48"/>
       <c r="F37" s="46"/>
       <c r="G37" s="49"/>
       <c r="H37" s="45"/>
       <c r="I37" s="50"/>
     </row>
-    <row r="38" spans="1:9" ht="13.5" customHeight="1">
+    <row r="38" spans="1:9" ht="15" customHeight="1">
       <c r="A38" s="44"/>
       <c r="B38" s="45"/>
-      <c r="C38" s="55"/>
-      <c r="D38" s="56"/>
+      <c r="C38" s="98"/>
+      <c r="D38" s="99"/>
       <c r="E38" s="48"/>
       <c r="F38" s="46"/>
       <c r="G38" s="49"/>
       <c r="H38" s="45"/>
       <c r="I38" s="50"/>
     </row>
-    <row r="39" spans="1:9" ht="13.7" customHeight="1">
+    <row r="39" spans="1:9" ht="15" customHeight="1">
       <c r="A39" s="44"/>
       <c r="B39" s="45"/>
-      <c r="C39" s="55"/>
-      <c r="D39" s="56"/>
+      <c r="C39" s="98"/>
+      <c r="D39" s="99"/>
       <c r="E39" s="48"/>
       <c r="F39" s="46"/>
       <c r="G39" s="49"/>
       <c r="H39" s="45"/>
       <c r="I39" s="50"/>
     </row>
-    <row r="40" spans="1:9" ht="13.7" customHeight="1">
+    <row r="40" spans="1:9" ht="15" customHeight="1">
       <c r="A40" s="44"/>
       <c r="B40" s="45"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="56"/>
+      <c r="C40" s="98"/>
+      <c r="D40" s="99"/>
       <c r="E40" s="48"/>
       <c r="F40" s="46"/>
       <c r="G40" s="49"/>
       <c r="H40" s="45"/>
       <c r="I40" s="50"/>
     </row>
-    <row r="41" spans="1:9" ht="13.7" customHeight="1">
+    <row r="41" spans="1:9" ht="15" customHeight="1">
       <c r="A41" s="44"/>
       <c r="B41" s="45"/>
-      <c r="C41" s="55"/>
-      <c r="D41" s="56"/>
+      <c r="C41" s="98"/>
+      <c r="D41" s="99"/>
       <c r="E41" s="48"/>
       <c r="F41" s="46"/>
       <c r="G41" s="49"/>
       <c r="H41" s="45"/>
       <c r="I41" s="50"/>
     </row>
-    <row r="42" spans="1:9" ht="13.7" customHeight="1">
+    <row r="42" spans="1:9" ht="15" customHeight="1">
       <c r="A42" s="44"/>
       <c r="B42" s="45"/>
-      <c r="C42" s="55"/>
-      <c r="D42" s="56"/>
+      <c r="C42" s="98"/>
+      <c r="D42" s="99"/>
       <c r="E42" s="48"/>
       <c r="F42" s="46"/>
       <c r="G42" s="49"/>
       <c r="H42" s="45"/>
       <c r="I42" s="50"/>
     </row>
-    <row r="43" spans="1:9" ht="13.7" customHeight="1">
+    <row r="43" spans="1:9" ht="15" customHeight="1">
       <c r="A43" s="44"/>
       <c r="B43" s="45"/>
-      <c r="C43" s="55"/>
-      <c r="D43" s="56"/>
+      <c r="C43" s="98"/>
+      <c r="D43" s="99"/>
       <c r="E43" s="48"/>
       <c r="F43" s="46"/>
       <c r="G43" s="49"/>
       <c r="H43" s="45"/>
       <c r="I43" s="50"/>
     </row>
-    <row r="44" spans="1:9" ht="13.7" customHeight="1">
+    <row r="44" spans="1:9" ht="15" customHeight="1">
       <c r="A44" s="44"/>
       <c r="B44" s="45"/>
-      <c r="C44" s="55"/>
-      <c r="D44" s="56"/>
+      <c r="C44" s="98"/>
+      <c r="D44" s="99"/>
       <c r="E44" s="48"/>
       <c r="F44" s="46"/>
       <c r="G44" s="49"/>
       <c r="H44" s="45"/>
       <c r="I44" s="50"/>
     </row>
-    <row r="45" spans="1:9" ht="13.7" customHeight="1">
+    <row r="45" spans="1:9" ht="15" customHeight="1">
       <c r="A45" s="44"/>
       <c r="B45" s="45"/>
-      <c r="C45" s="55"/>
-      <c r="D45" s="56"/>
+      <c r="C45" s="98"/>
+      <c r="D45" s="99"/>
       <c r="E45" s="48"/>
       <c r="F45" s="46"/>
       <c r="G45" s="49"/>
       <c r="H45" s="45"/>
       <c r="I45" s="50"/>
     </row>
-    <row r="46" spans="1:9" ht="13.7" customHeight="1">
+    <row r="46" spans="1:9" ht="15" customHeight="1">
       <c r="A46" s="44"/>
       <c r="B46" s="45"/>
-      <c r="C46" s="55"/>
-      <c r="D46" s="56"/>
+      <c r="C46" s="98"/>
+      <c r="D46" s="99"/>
       <c r="E46" s="48"/>
       <c r="F46" s="46"/>
       <c r="G46" s="49"/>
       <c r="H46" s="45"/>
       <c r="I46" s="50"/>
     </row>
-    <row r="47" spans="1:9" ht="13.7" customHeight="1">
+    <row r="47" spans="1:9" ht="15" customHeight="1">
       <c r="A47" s="44"/>
       <c r="B47" s="45"/>
-      <c r="C47" s="55"/>
-      <c r="D47" s="56"/>
+      <c r="C47" s="98"/>
+      <c r="D47" s="99"/>
       <c r="E47" s="48"/>
       <c r="F47" s="46"/>
       <c r="G47" s="49"/>
       <c r="H47" s="45"/>
       <c r="I47" s="50"/>
     </row>
-    <row r="48" spans="1:9" ht="13.7" customHeight="1">
+    <row r="48" spans="1:9" ht="15" customHeight="1">
       <c r="A48" s="44"/>
       <c r="B48" s="45"/>
-      <c r="C48" s="55"/>
-      <c r="D48" s="56"/>
+      <c r="C48" s="98"/>
+      <c r="D48" s="99"/>
       <c r="E48" s="48"/>
       <c r="F48" s="46"/>
       <c r="G48" s="49"/>
       <c r="H48" s="45"/>
       <c r="I48" s="50"/>
     </row>
-    <row r="49" spans="1:9" ht="13.7" customHeight="1">
+    <row r="49" spans="1:9" ht="15" customHeight="1">
       <c r="A49" s="44"/>
       <c r="B49" s="45"/>
-      <c r="C49" s="55"/>
-      <c r="D49" s="56"/>
+      <c r="C49" s="98"/>
+      <c r="D49" s="99"/>
       <c r="E49" s="48"/>
       <c r="F49" s="46"/>
       <c r="G49" s="49"/>
       <c r="H49" s="45"/>
       <c r="I49" s="50"/>
     </row>
-    <row r="50" spans="1:9" ht="13.7" hidden="1" customHeight="1">
+    <row r="50" spans="1:9" ht="15" customHeight="1">
       <c r="A50" s="44"/>
       <c r="B50" s="45"/>
-      <c r="C50" s="55"/>
-      <c r="D50" s="56"/>
+      <c r="C50" s="98"/>
+      <c r="D50" s="99"/>
       <c r="E50" s="48"/>
       <c r="F50" s="46"/>
       <c r="G50" s="49"/>
       <c r="H50" s="45"/>
       <c r="I50" s="50"/>
     </row>
-    <row r="51" spans="1:9" ht="13.7" customHeight="1">
+    <row r="51" spans="1:9" ht="15" customHeight="1">
       <c r="A51" s="44"/>
       <c r="B51" s="45"/>
-      <c r="C51" s="55"/>
-      <c r="D51" s="56"/>
+      <c r="C51" s="98"/>
+      <c r="D51" s="99"/>
       <c r="E51" s="48"/>
       <c r="F51" s="46"/>
       <c r="G51" s="49"/>
       <c r="H51" s="45"/>
       <c r="I51" s="50"/>
     </row>
-    <row r="52" spans="1:9" ht="13.7" customHeight="1">
+    <row r="52" spans="1:9" ht="15" customHeight="1">
       <c r="A52" s="44"/>
       <c r="B52" s="45"/>
-      <c r="C52" s="55"/>
-      <c r="D52" s="56"/>
+      <c r="C52" s="98"/>
+      <c r="D52" s="99"/>
       <c r="E52" s="48"/>
       <c r="F52" s="46"/>
       <c r="G52" s="49"/>
       <c r="H52" s="45"/>
       <c r="I52" s="50"/>
     </row>
-    <row r="53" spans="1:9" ht="13.7" customHeight="1">
+    <row r="53" spans="1:9" ht="15" customHeight="1">
       <c r="A53" s="44"/>
       <c r="B53" s="45"/>
-      <c r="C53" s="55"/>
-      <c r="D53" s="56"/>
+      <c r="C53" s="98"/>
+      <c r="D53" s="99"/>
       <c r="E53" s="48"/>
       <c r="F53" s="46"/>
       <c r="G53" s="49"/>
       <c r="H53" s="45"/>
       <c r="I53" s="50"/>
     </row>
-    <row r="54" spans="1:9" ht="13.7" customHeight="1">
+    <row r="54" spans="1:9" ht="15" customHeight="1">
       <c r="A54" s="44"/>
       <c r="B54" s="45"/>
-      <c r="C54" s="55"/>
-      <c r="D54" s="56"/>
+      <c r="C54" s="98"/>
+      <c r="D54" s="99"/>
       <c r="E54" s="48"/>
       <c r="F54" s="46"/>
       <c r="G54" s="49"/>
       <c r="H54" s="45"/>
       <c r="I54" s="50"/>
     </row>
-    <row r="55" spans="1:9" ht="13.7" customHeight="1">
+    <row r="55" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A55" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="B55" s="73"/>
-      <c r="C55" s="73"/>
-      <c r="D55" s="73"/>
-      <c r="E55" s="73"/>
-      <c r="F55" s="73"/>
-      <c r="G55" s="73"/>
-      <c r="H55" s="73"/>
-      <c r="I55" s="74"/>
-    </row>
-    <row r="56" spans="1:9" ht="13.7" customHeight="1">
+      <c r="B55" s="102"/>
+      <c r="C55" s="102"/>
+      <c r="D55" s="102"/>
+      <c r="E55" s="102"/>
+      <c r="F55" s="102"/>
+      <c r="G55" s="102"/>
+      <c r="H55" s="102"/>
+      <c r="I55" s="103"/>
+    </row>
+    <row r="56" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A56" s="32"/>
-      <c r="B56" s="75"/>
-      <c r="C56" s="75"/>
-      <c r="D56" s="75"/>
-      <c r="E56" s="75"/>
-      <c r="F56" s="75"/>
-      <c r="G56" s="75"/>
-      <c r="H56" s="75"/>
-      <c r="I56" s="76"/>
-    </row>
-    <row r="57" spans="1:9" ht="13.7" customHeight="1">
-      <c r="A57" s="77"/>
-      <c r="B57" s="78"/>
+      <c r="B56" s="104"/>
+      <c r="C56" s="104"/>
+      <c r="D56" s="104"/>
+      <c r="E56" s="104"/>
+      <c r="F56" s="104"/>
+      <c r="G56" s="104"/>
+      <c r="H56" s="104"/>
+      <c r="I56" s="105"/>
+    </row>
+    <row r="57" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A57" s="106"/>
+      <c r="B57" s="107"/>
       <c r="C57" s="53" t="s">
         <v>24</v>
       </c>
       <c r="D57" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E57" s="68" t="s">
+      <c r="E57" s="108" t="s">
         <v>26</v>
       </c>
-      <c r="F57" s="79"/>
-      <c r="G57" s="69"/>
-      <c r="H57" s="68" t="s">
+      <c r="F57" s="109"/>
+      <c r="G57" s="110"/>
+      <c r="H57" s="108" t="s">
         <v>27</v>
       </c>
-      <c r="I57" s="69"/>
-    </row>
-    <row r="58" spans="1:9" ht="13.7" customHeight="1">
-      <c r="A58" s="68" t="s">
+      <c r="I57" s="110"/>
+    </row>
+    <row r="58" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A58" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="B58" s="69"/>
+      <c r="B58" s="110"/>
       <c r="C58" s="54"/>
       <c r="D58" s="54"/>
-      <c r="E58" s="70"/>
-      <c r="F58" s="71"/>
-      <c r="G58" s="72"/>
-      <c r="H58" s="70"/>
-      <c r="I58" s="72"/>
-    </row>
-    <row r="59" spans="1:9" ht="13.7" customHeight="1">
-      <c r="A59" s="68" t="s">
+      <c r="E58" s="111"/>
+      <c r="F58" s="112"/>
+      <c r="G58" s="113"/>
+      <c r="H58" s="111"/>
+      <c r="I58" s="113"/>
+    </row>
+    <row r="59" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A59" s="108" t="s">
         <v>29</v>
       </c>
-      <c r="B59" s="69"/>
-      <c r="C59" s="158"/>
-      <c r="D59" s="159"/>
-      <c r="E59" s="160"/>
-      <c r="F59" s="161"/>
-      <c r="G59" s="162"/>
-      <c r="H59" s="160"/>
-      <c r="I59" s="162"/>
-    </row>
-    <row r="60" spans="1:9" ht="13.7" customHeight="1">
-      <c r="A60" s="65" t="s">
+      <c r="B59" s="110"/>
+      <c r="C59" s="56"/>
+      <c r="D59" s="57"/>
+      <c r="E59" s="114"/>
+      <c r="F59" s="115"/>
+      <c r="G59" s="116"/>
+      <c r="H59" s="114"/>
+      <c r="I59" s="116"/>
+    </row>
+    <row r="60" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A60" s="117" t="s">
         <v>30</v>
       </c>
-      <c r="B60" s="65"/>
-      <c r="C60" s="155"/>
-      <c r="D60" s="155"/>
-      <c r="E60" s="156"/>
-      <c r="F60" s="156"/>
-      <c r="G60" s="156"/>
-      <c r="H60" s="157"/>
-      <c r="I60" s="157"/>
-    </row>
-    <row r="61" spans="1:9" ht="13.7" customHeight="1">
-      <c r="A61" s="65" t="s">
+      <c r="B60" s="117"/>
+      <c r="C60" s="55"/>
+      <c r="D60" s="55"/>
+      <c r="E60" s="118"/>
+      <c r="F60" s="118"/>
+      <c r="G60" s="118"/>
+      <c r="H60" s="119"/>
+      <c r="I60" s="119"/>
+    </row>
+    <row r="61" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A61" s="117" t="s">
         <v>31</v>
       </c>
-      <c r="B61" s="65"/>
+      <c r="B61" s="117"/>
       <c r="C61" s="52"/>
       <c r="D61" s="52"/>
-      <c r="E61" s="66"/>
-      <c r="F61" s="66"/>
-      <c r="G61" s="66"/>
-      <c r="H61" s="67"/>
-      <c r="I61" s="67"/>
+      <c r="E61" s="120"/>
+      <c r="F61" s="120"/>
+      <c r="G61" s="120"/>
+      <c r="H61" s="121"/>
+      <c r="I61" s="121"/>
+    </row>
+    <row r="62" spans="1:9">
+      <c r="A62" s="171"/>
+      <c r="B62" s="172" t="s">
+        <v>53</v>
+      </c>
+      <c r="C62" s="170"/>
+    </row>
+    <row r="63" spans="1:9" ht="15" customHeight="1">
+      <c r="C63" s="170"/>
     </row>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:I1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:I2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:I4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:I6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="C53:D53"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="C50:D50"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="E60:G60"/>
+    <mergeCell ref="H60:I60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="H58:I58"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="B56:I56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="H57:I57"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="C20:D20"/>
@@ -2205,40 +2275,40 @@
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="B55:I55"/>
-    <mergeCell ref="B56:I56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="E57:G57"/>
-    <mergeCell ref="H57:I57"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="E58:G58"/>
-    <mergeCell ref="H58:I58"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="E59:G59"/>
-    <mergeCell ref="H59:I59"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="E60:G60"/>
-    <mergeCell ref="H60:I60"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="H61:I61"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="C53:D53"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:I3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -2261,117 +2331,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="108"/>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="110"/>
-      <c r="E1" s="111"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="113"/>
+      <c r="A1" s="58"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="63"/>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A2" s="153" t="s">
+      <c r="A2" s="130" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="115"/>
-      <c r="C2" s="115"/>
-      <c r="D2" s="116"/>
-      <c r="E2" s="117"/>
-      <c r="F2" s="118"/>
-      <c r="G2" s="118"/>
-      <c r="H2" s="118"/>
-      <c r="I2" s="119"/>
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="69"/>
     </row>
     <row r="3" spans="1:9" ht="17.25" customHeight="1">
-      <c r="A3" s="153" t="s">
+      <c r="A3" s="130" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="115"/>
-      <c r="C3" s="115"/>
-      <c r="D3" s="116"/>
-      <c r="E3" s="154" t="s">
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="131" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="121"/>
-      <c r="G3" s="121"/>
-      <c r="H3" s="121"/>
-      <c r="I3" s="122"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="72"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="151" t="s">
+      <c r="A4" s="132" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="96"/>
-      <c r="C4" s="96"/>
-      <c r="D4" s="97"/>
-      <c r="E4" s="101" t="s">
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="75"/>
+      <c r="E4" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="99"/>
-      <c r="G4" s="99"/>
-      <c r="H4" s="99"/>
-      <c r="I4" s="100"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
+      <c r="I4" s="78"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="151" t="s">
+      <c r="A5" s="132" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="96"/>
-      <c r="C5" s="96"/>
-      <c r="D5" s="97"/>
-      <c r="E5" s="101"/>
-      <c r="F5" s="99"/>
-      <c r="G5" s="99"/>
-      <c r="H5" s="99"/>
-      <c r="I5" s="100"/>
+      <c r="B5" s="74"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="75"/>
+      <c r="E5" s="79"/>
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="77"/>
+      <c r="I5" s="78"/>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="152" t="s">
+      <c r="A6" s="133" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="103"/>
-      <c r="C6" s="103"/>
-      <c r="D6" s="104"/>
-      <c r="E6" s="105"/>
-      <c r="F6" s="106"/>
-      <c r="G6" s="106"/>
-      <c r="H6" s="106"/>
-      <c r="I6" s="107"/>
+      <c r="B6" s="81"/>
+      <c r="C6" s="81"/>
+      <c r="D6" s="82"/>
+      <c r="E6" s="83"/>
+      <c r="F6" s="84"/>
+      <c r="G6" s="84"/>
+      <c r="H6" s="84"/>
+      <c r="I6" s="85"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="144" t="s">
+      <c r="A7" s="134" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="125" t="s">
+      <c r="B7" s="86"/>
+      <c r="C7" s="160" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="126" t="s">
+      <c r="D7" s="161" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="63"/>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64"/>
-      <c r="H7" s="64"/>
+      <c r="E7" s="128"/>
+      <c r="F7" s="129"/>
+      <c r="G7" s="129"/>
+      <c r="H7" s="129"/>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="145" t="s">
+      <c r="B8" s="135" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="145"/>
-      <c r="D8" s="146"/>
-      <c r="E8" s="63" t="s">
+      <c r="C8" s="135"/>
+      <c r="D8" s="136"/>
+      <c r="E8" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="64"/>
-      <c r="G8" s="64"/>
-      <c r="H8" s="64"/>
+      <c r="F8" s="129"/>
+      <c r="G8" s="129"/>
+      <c r="H8" s="129"/>
       <c r="I8" s="3" t="s">
         <v>34</v>
       </c>
@@ -2380,37 +2450,37 @@
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="145" t="s">
+      <c r="B9" s="135" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="145"/>
-      <c r="D9" s="146"/>
-      <c r="E9" s="63" t="s">
+      <c r="C9" s="135"/>
+      <c r="D9" s="136"/>
+      <c r="E9" s="128" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="64"/>
-      <c r="G9" s="147" t="s">
+      <c r="F9" s="129"/>
+      <c r="G9" s="137" t="s">
         <v>36</v>
       </c>
-      <c r="H9" s="147"/>
-      <c r="I9" s="148"/>
+      <c r="H9" s="137"/>
+      <c r="I9" s="138"/>
     </row>
     <row r="10" spans="1:9" ht="15" customHeight="1">
-      <c r="A10" s="149" t="s">
+      <c r="A10" s="139" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="91"/>
-      <c r="C10" s="91"/>
-      <c r="D10" s="91"/>
-      <c r="E10" s="92"/>
-      <c r="F10" s="150" t="s">
+      <c r="B10" s="94"/>
+      <c r="C10" s="94"/>
+      <c r="D10" s="94"/>
+      <c r="E10" s="95"/>
+      <c r="F10" s="140" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="94"/>
-      <c r="H10" s="149" t="s">
+      <c r="G10" s="97"/>
+      <c r="H10" s="139" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="92"/>
+      <c r="I10" s="95"/>
     </row>
     <row r="11" spans="1:9" ht="30" customHeight="1">
       <c r="A11" s="4" t="s">
@@ -2419,10 +2489,10 @@
       <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="135" t="s">
+      <c r="C11" s="143" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="81"/>
+      <c r="D11" s="101"/>
       <c r="E11" s="5" t="s">
         <v>19</v>
       </c>
@@ -2446,10 +2516,10 @@
       <c r="B12" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="123" t="s">
+      <c r="C12" s="141" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="124"/>
+      <c r="D12" s="142"/>
       <c r="E12" s="7" t="s">
         <v>40</v>
       </c>
@@ -2469,8 +2539,8 @@
     <row r="13" spans="1:9" ht="13.7" customHeight="1">
       <c r="A13" s="4"/>
       <c r="B13" s="6"/>
-      <c r="C13" s="123"/>
-      <c r="D13" s="124"/>
+      <c r="C13" s="141"/>
+      <c r="D13" s="142"/>
       <c r="E13" s="11"/>
       <c r="F13" s="8"/>
       <c r="G13" s="9"/>
@@ -2480,8 +2550,8 @@
     <row r="14" spans="1:9" ht="13.7" customHeight="1">
       <c r="A14" s="4"/>
       <c r="B14" s="6"/>
-      <c r="C14" s="123"/>
-      <c r="D14" s="124"/>
+      <c r="C14" s="141"/>
+      <c r="D14" s="142"/>
       <c r="E14" s="11"/>
       <c r="F14" s="8"/>
       <c r="G14" s="9"/>
@@ -2491,8 +2561,8 @@
     <row r="15" spans="1:9" ht="13.7" customHeight="1">
       <c r="A15" s="4"/>
       <c r="B15" s="6"/>
-      <c r="C15" s="123"/>
-      <c r="D15" s="124"/>
+      <c r="C15" s="141"/>
+      <c r="D15" s="142"/>
       <c r="E15" s="13"/>
       <c r="F15" s="8"/>
       <c r="G15" s="9"/>
@@ -2502,8 +2572,8 @@
     <row r="16" spans="1:9" ht="13.7" customHeight="1">
       <c r="A16" s="4"/>
       <c r="B16" s="6"/>
-      <c r="C16" s="123"/>
-      <c r="D16" s="124"/>
+      <c r="C16" s="141"/>
+      <c r="D16" s="142"/>
       <c r="E16" s="13"/>
       <c r="F16" s="8"/>
       <c r="G16" s="9"/>
@@ -2513,8 +2583,8 @@
     <row r="17" spans="1:9" ht="13.7" customHeight="1">
       <c r="A17" s="4"/>
       <c r="B17" s="6"/>
-      <c r="C17" s="123"/>
-      <c r="D17" s="124"/>
+      <c r="C17" s="141"/>
+      <c r="D17" s="142"/>
       <c r="E17" s="13"/>
       <c r="F17" s="8"/>
       <c r="G17" s="9"/>
@@ -2524,8 +2594,8 @@
     <row r="18" spans="1:9" ht="13.7" customHeight="1">
       <c r="A18" s="4"/>
       <c r="B18" s="6"/>
-      <c r="C18" s="123"/>
-      <c r="D18" s="124"/>
+      <c r="C18" s="141"/>
+      <c r="D18" s="142"/>
       <c r="E18" s="13"/>
       <c r="F18" s="8"/>
       <c r="G18" s="9"/>
@@ -2535,8 +2605,8 @@
     <row r="19" spans="1:9" ht="13.7" customHeight="1">
       <c r="A19" s="15"/>
       <c r="B19" s="6"/>
-      <c r="C19" s="123"/>
-      <c r="D19" s="124"/>
+      <c r="C19" s="141"/>
+      <c r="D19" s="142"/>
       <c r="E19" s="16"/>
       <c r="F19" s="8"/>
       <c r="G19" s="9"/>
@@ -2546,8 +2616,8 @@
     <row r="20" spans="1:9" ht="13.7" customHeight="1">
       <c r="A20" s="15"/>
       <c r="B20" s="6"/>
-      <c r="C20" s="123"/>
-      <c r="D20" s="124"/>
+      <c r="C20" s="141"/>
+      <c r="D20" s="142"/>
       <c r="E20" s="16"/>
       <c r="F20" s="8"/>
       <c r="G20" s="9"/>
@@ -2557,8 +2627,8 @@
     <row r="21" spans="1:9" ht="13.7" customHeight="1">
       <c r="A21" s="15"/>
       <c r="B21" s="6"/>
-      <c r="C21" s="123"/>
-      <c r="D21" s="124"/>
+      <c r="C21" s="141"/>
+      <c r="D21" s="142"/>
       <c r="E21" s="16"/>
       <c r="F21" s="8"/>
       <c r="G21" s="9"/>
@@ -2568,8 +2638,8 @@
     <row r="22" spans="1:9" ht="13.7" customHeight="1">
       <c r="A22" s="18"/>
       <c r="B22" s="6"/>
-      <c r="C22" s="123"/>
-      <c r="D22" s="124"/>
+      <c r="C22" s="141"/>
+      <c r="D22" s="142"/>
       <c r="E22" s="19"/>
       <c r="F22" s="20"/>
       <c r="G22" s="21"/>
@@ -2579,8 +2649,8 @@
     <row r="23" spans="1:9" ht="13.7" customHeight="1">
       <c r="A23" s="18"/>
       <c r="B23" s="6"/>
-      <c r="C23" s="123"/>
-      <c r="D23" s="124"/>
+      <c r="C23" s="141"/>
+      <c r="D23" s="142"/>
       <c r="E23" s="19"/>
       <c r="F23" s="22"/>
       <c r="G23" s="21"/>
@@ -2590,8 +2660,8 @@
     <row r="24" spans="1:9" ht="13.7" customHeight="1">
       <c r="A24" s="18"/>
       <c r="B24" s="6"/>
-      <c r="C24" s="123"/>
-      <c r="D24" s="124"/>
+      <c r="C24" s="141"/>
+      <c r="D24" s="142"/>
       <c r="E24" s="19"/>
       <c r="F24" s="22"/>
       <c r="G24" s="21"/>
@@ -2601,8 +2671,8 @@
     <row r="25" spans="1:9" ht="13.7" customHeight="1">
       <c r="A25" s="18"/>
       <c r="B25" s="6"/>
-      <c r="C25" s="123"/>
-      <c r="D25" s="124"/>
+      <c r="C25" s="141"/>
+      <c r="D25" s="142"/>
       <c r="E25" s="19"/>
       <c r="F25" s="22"/>
       <c r="G25" s="21"/>
@@ -2612,8 +2682,8 @@
     <row r="26" spans="1:9" ht="13.7" customHeight="1">
       <c r="A26" s="18"/>
       <c r="B26" s="6"/>
-      <c r="C26" s="123"/>
-      <c r="D26" s="124"/>
+      <c r="C26" s="141"/>
+      <c r="D26" s="142"/>
       <c r="E26" s="19"/>
       <c r="F26" s="22"/>
       <c r="G26" s="21"/>
@@ -2623,8 +2693,8 @@
     <row r="27" spans="1:9" ht="13.7" customHeight="1">
       <c r="A27" s="18"/>
       <c r="B27" s="6"/>
-      <c r="C27" s="123"/>
-      <c r="D27" s="124"/>
+      <c r="C27" s="141"/>
+      <c r="D27" s="142"/>
       <c r="E27" s="19"/>
       <c r="F27" s="22"/>
       <c r="G27" s="21"/>
@@ -2634,8 +2704,8 @@
     <row r="28" spans="1:9" ht="13.7" customHeight="1">
       <c r="A28" s="18"/>
       <c r="B28" s="6"/>
-      <c r="C28" s="123"/>
-      <c r="D28" s="124"/>
+      <c r="C28" s="141"/>
+      <c r="D28" s="142"/>
       <c r="E28" s="19"/>
       <c r="F28" s="22"/>
       <c r="G28" s="21"/>
@@ -2645,8 +2715,8 @@
     <row r="29" spans="1:9" ht="13.7" customHeight="1">
       <c r="A29" s="15"/>
       <c r="B29" s="6"/>
-      <c r="C29" s="123"/>
-      <c r="D29" s="124"/>
+      <c r="C29" s="141"/>
+      <c r="D29" s="142"/>
       <c r="E29" s="19"/>
       <c r="F29" s="8"/>
       <c r="G29" s="9"/>
@@ -2656,8 +2726,8 @@
     <row r="30" spans="1:9" ht="13.7" customHeight="1">
       <c r="A30" s="15"/>
       <c r="B30" s="6"/>
-      <c r="C30" s="123"/>
-      <c r="D30" s="124"/>
+      <c r="C30" s="141"/>
+      <c r="D30" s="142"/>
       <c r="E30" s="19"/>
       <c r="F30" s="8"/>
       <c r="G30" s="9"/>
@@ -2667,8 +2737,8 @@
     <row r="31" spans="1:9" ht="13.7" customHeight="1">
       <c r="A31" s="15"/>
       <c r="B31" s="6"/>
-      <c r="C31" s="123"/>
-      <c r="D31" s="124"/>
+      <c r="C31" s="141"/>
+      <c r="D31" s="142"/>
       <c r="E31" s="19"/>
       <c r="F31" s="8"/>
       <c r="G31" s="9"/>
@@ -2678,8 +2748,8 @@
     <row r="32" spans="1:9" ht="13.7" customHeight="1">
       <c r="A32" s="15"/>
       <c r="B32" s="6"/>
-      <c r="C32" s="123"/>
-      <c r="D32" s="124"/>
+      <c r="C32" s="141"/>
+      <c r="D32" s="142"/>
       <c r="E32" s="19"/>
       <c r="F32" s="8"/>
       <c r="G32" s="9"/>
@@ -2689,8 +2759,8 @@
     <row r="33" spans="1:15" ht="13.7" customHeight="1">
       <c r="A33" s="15"/>
       <c r="B33" s="6"/>
-      <c r="C33" s="123"/>
-      <c r="D33" s="124"/>
+      <c r="C33" s="141"/>
+      <c r="D33" s="142"/>
       <c r="E33" s="19"/>
       <c r="F33" s="25"/>
       <c r="G33" s="9"/>
@@ -2700,8 +2770,8 @@
     <row r="34" spans="1:15" ht="13.7" customHeight="1">
       <c r="A34" s="15"/>
       <c r="B34" s="6"/>
-      <c r="C34" s="123"/>
-      <c r="D34" s="124"/>
+      <c r="C34" s="141"/>
+      <c r="D34" s="142"/>
       <c r="E34" s="19"/>
       <c r="F34" s="26"/>
       <c r="G34" s="9"/>
@@ -2711,8 +2781,8 @@
     <row r="35" spans="1:15" ht="13.7" customHeight="1">
       <c r="A35" s="15"/>
       <c r="B35" s="6"/>
-      <c r="C35" s="123"/>
-      <c r="D35" s="124"/>
+      <c r="C35" s="141"/>
+      <c r="D35" s="142"/>
       <c r="E35" s="19"/>
       <c r="F35" s="26"/>
       <c r="G35" s="9"/>
@@ -2722,8 +2792,8 @@
     <row r="36" spans="1:15" ht="13.7" customHeight="1">
       <c r="A36" s="15"/>
       <c r="B36" s="6"/>
-      <c r="C36" s="123"/>
-      <c r="D36" s="124"/>
+      <c r="C36" s="141"/>
+      <c r="D36" s="142"/>
       <c r="E36" s="19"/>
       <c r="F36" s="26"/>
       <c r="G36" s="9"/>
@@ -2733,8 +2803,8 @@
     <row r="37" spans="1:15" ht="13.7" customHeight="1">
       <c r="A37" s="15"/>
       <c r="B37" s="27"/>
-      <c r="C37" s="123"/>
-      <c r="D37" s="124"/>
+      <c r="C37" s="141"/>
+      <c r="D37" s="142"/>
       <c r="E37" s="19"/>
       <c r="F37" s="26"/>
       <c r="G37" s="9"/>
@@ -2744,8 +2814,8 @@
     <row r="38" spans="1:15" ht="13.7" customHeight="1">
       <c r="A38" s="15"/>
       <c r="B38" s="6"/>
-      <c r="C38" s="123"/>
-      <c r="D38" s="124"/>
+      <c r="C38" s="141"/>
+      <c r="D38" s="142"/>
       <c r="E38" s="7"/>
       <c r="F38" s="26"/>
       <c r="G38" s="9"/>
@@ -2758,8 +2828,8 @@
     <row r="39" spans="1:15" ht="13.7" customHeight="1">
       <c r="A39" s="15"/>
       <c r="B39" s="6"/>
-      <c r="C39" s="123"/>
-      <c r="D39" s="124"/>
+      <c r="C39" s="141"/>
+      <c r="D39" s="142"/>
       <c r="E39" s="28"/>
       <c r="F39" s="26"/>
       <c r="G39" s="9"/>
@@ -2769,8 +2839,8 @@
     <row r="40" spans="1:15" ht="13.7" customHeight="1">
       <c r="A40" s="15"/>
       <c r="B40" s="6"/>
-      <c r="C40" s="123"/>
-      <c r="D40" s="124"/>
+      <c r="C40" s="141"/>
+      <c r="D40" s="142"/>
       <c r="E40" s="28"/>
       <c r="F40" s="26"/>
       <c r="G40" s="9"/>
@@ -2780,8 +2850,8 @@
     <row r="41" spans="1:15" ht="13.7" customHeight="1">
       <c r="A41" s="15"/>
       <c r="B41" s="6"/>
-      <c r="C41" s="123"/>
-      <c r="D41" s="124"/>
+      <c r="C41" s="141"/>
+      <c r="D41" s="142"/>
       <c r="E41" s="28"/>
       <c r="F41" s="26"/>
       <c r="G41" s="9"/>
@@ -2791,8 +2861,8 @@
     <row r="42" spans="1:15" ht="13.7" customHeight="1">
       <c r="A42" s="15"/>
       <c r="B42" s="6"/>
-      <c r="C42" s="123"/>
-      <c r="D42" s="124"/>
+      <c r="C42" s="141"/>
+      <c r="D42" s="142"/>
       <c r="E42" s="28"/>
       <c r="F42" s="26"/>
       <c r="G42" s="9"/>
@@ -2802,8 +2872,8 @@
     <row r="43" spans="1:15" ht="13.7" customHeight="1">
       <c r="A43" s="15"/>
       <c r="B43" s="6"/>
-      <c r="C43" s="123"/>
-      <c r="D43" s="124"/>
+      <c r="C43" s="141"/>
+      <c r="D43" s="142"/>
       <c r="E43" s="28"/>
       <c r="F43" s="26"/>
       <c r="G43" s="9"/>
@@ -2816,8 +2886,8 @@
     <row r="44" spans="1:15" ht="13.7" customHeight="1">
       <c r="A44" s="15"/>
       <c r="B44" s="6"/>
-      <c r="C44" s="123"/>
-      <c r="D44" s="124"/>
+      <c r="C44" s="141"/>
+      <c r="D44" s="142"/>
       <c r="E44" s="28"/>
       <c r="F44" s="26"/>
       <c r="G44" s="9"/>
@@ -2827,8 +2897,8 @@
     <row r="45" spans="1:15" ht="13.7" customHeight="1">
       <c r="A45" s="15"/>
       <c r="B45" s="6"/>
-      <c r="C45" s="123"/>
-      <c r="D45" s="124"/>
+      <c r="C45" s="141"/>
+      <c r="D45" s="142"/>
       <c r="E45" s="28"/>
       <c r="F45" s="26"/>
       <c r="G45" s="9"/>
@@ -2838,8 +2908,8 @@
     <row r="46" spans="1:15" ht="13.7" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="6"/>
-      <c r="C46" s="123"/>
-      <c r="D46" s="124"/>
+      <c r="C46" s="141"/>
+      <c r="D46" s="142"/>
       <c r="E46" s="8"/>
       <c r="F46" s="26"/>
       <c r="G46" s="9"/>
@@ -2849,8 +2919,8 @@
     <row r="47" spans="1:15" ht="13.7" customHeight="1">
       <c r="A47" s="15"/>
       <c r="B47" s="6"/>
-      <c r="C47" s="123"/>
-      <c r="D47" s="124"/>
+      <c r="C47" s="141"/>
+      <c r="D47" s="142"/>
       <c r="E47" s="28"/>
       <c r="F47" s="26"/>
       <c r="G47" s="9"/>
@@ -2860,8 +2930,8 @@
     <row r="48" spans="1:15" ht="13.7" customHeight="1">
       <c r="A48" s="15"/>
       <c r="B48" s="6"/>
-      <c r="C48" s="123"/>
-      <c r="D48" s="124"/>
+      <c r="C48" s="141"/>
+      <c r="D48" s="142"/>
       <c r="E48" s="28"/>
       <c r="F48" s="26"/>
       <c r="G48" s="9"/>
@@ -2871,8 +2941,8 @@
     <row r="49" spans="1:13" ht="13.7" customHeight="1">
       <c r="A49" s="15"/>
       <c r="B49" s="29"/>
-      <c r="C49" s="123"/>
-      <c r="D49" s="124"/>
+      <c r="C49" s="141"/>
+      <c r="D49" s="142"/>
       <c r="E49" s="28"/>
       <c r="F49" s="26"/>
       <c r="G49" s="9"/>
@@ -2882,8 +2952,8 @@
     <row r="50" spans="1:13" ht="13.7" hidden="1" customHeight="1">
       <c r="A50" s="15"/>
       <c r="B50" s="6"/>
-      <c r="C50" s="123"/>
-      <c r="D50" s="124"/>
+      <c r="C50" s="141"/>
+      <c r="D50" s="142"/>
       <c r="E50" s="28"/>
       <c r="F50" s="26"/>
       <c r="G50" s="9"/>
@@ -2893,8 +2963,8 @@
     <row r="51" spans="1:13" ht="13.7" customHeight="1">
       <c r="A51" s="15"/>
       <c r="B51" s="6"/>
-      <c r="C51" s="123"/>
-      <c r="D51" s="124"/>
+      <c r="C51" s="141"/>
+      <c r="D51" s="142"/>
       <c r="E51" s="28"/>
       <c r="F51" s="26"/>
       <c r="G51" s="9"/>
@@ -2904,8 +2974,8 @@
     <row r="52" spans="1:13" ht="13.7" customHeight="1">
       <c r="A52" s="15"/>
       <c r="B52" s="29"/>
-      <c r="C52" s="123"/>
-      <c r="D52" s="124"/>
+      <c r="C52" s="141"/>
+      <c r="D52" s="142"/>
       <c r="E52" s="28"/>
       <c r="F52" s="26"/>
       <c r="G52" s="9"/>
@@ -2915,8 +2985,8 @@
     <row r="53" spans="1:13" ht="13.7" customHeight="1">
       <c r="A53" s="15"/>
       <c r="B53" s="6"/>
-      <c r="C53" s="123"/>
-      <c r="D53" s="124"/>
+      <c r="C53" s="141"/>
+      <c r="D53" s="142"/>
       <c r="E53" s="28"/>
       <c r="F53" s="26"/>
       <c r="G53" s="9"/>
@@ -2926,8 +2996,8 @@
     <row r="54" spans="1:13" ht="13.7" customHeight="1">
       <c r="A54" s="15"/>
       <c r="B54" s="29"/>
-      <c r="C54" s="123"/>
-      <c r="D54" s="124"/>
+      <c r="C54" s="141"/>
+      <c r="D54" s="142"/>
       <c r="E54" s="28"/>
       <c r="F54" s="26"/>
       <c r="G54" s="9"/>
@@ -2938,113 +3008,116 @@
       <c r="A55" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="B55" s="141" t="s">
+      <c r="B55" s="144" t="s">
         <v>45</v>
       </c>
-      <c r="C55" s="141"/>
-      <c r="D55" s="141"/>
-      <c r="E55" s="141"/>
-      <c r="F55" s="141"/>
-      <c r="G55" s="141"/>
-      <c r="H55" s="141"/>
-      <c r="I55" s="142"/>
+      <c r="C55" s="144"/>
+      <c r="D55" s="144"/>
+      <c r="E55" s="144"/>
+      <c r="F55" s="144"/>
+      <c r="G55" s="144"/>
+      <c r="H55" s="144"/>
+      <c r="I55" s="145"/>
     </row>
     <row r="56" spans="1:13" ht="13.7" customHeight="1">
       <c r="A56" s="32"/>
-      <c r="B56" s="75"/>
-      <c r="C56" s="75"/>
-      <c r="D56" s="75"/>
-      <c r="E56" s="75"/>
-      <c r="F56" s="75"/>
-      <c r="G56" s="75"/>
-      <c r="H56" s="75"/>
-      <c r="I56" s="76"/>
+      <c r="B56" s="104"/>
+      <c r="C56" s="104"/>
+      <c r="D56" s="104"/>
+      <c r="E56" s="104"/>
+      <c r="F56" s="104"/>
+      <c r="G56" s="104"/>
+      <c r="H56" s="104"/>
+      <c r="I56" s="105"/>
     </row>
     <row r="57" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A57" s="130"/>
-      <c r="B57" s="131"/>
+      <c r="A57" s="146"/>
+      <c r="B57" s="147"/>
       <c r="C57" s="33" t="s">
         <v>24</v>
       </c>
       <c r="D57" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="E57" s="130" t="s">
+      <c r="E57" s="146" t="s">
         <v>26</v>
       </c>
-      <c r="F57" s="143"/>
-      <c r="G57" s="131"/>
-      <c r="H57" s="130" t="s">
+      <c r="F57" s="148"/>
+      <c r="G57" s="147"/>
+      <c r="H57" s="146" t="s">
         <v>27</v>
       </c>
-      <c r="I57" s="131"/>
+      <c r="I57" s="147"/>
     </row>
     <row r="58" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A58" s="130" t="s">
+      <c r="A58" s="146" t="s">
         <v>28</v>
       </c>
-      <c r="B58" s="131"/>
+      <c r="B58" s="147"/>
       <c r="C58" s="34"/>
       <c r="D58" s="34"/>
-      <c r="E58" s="132"/>
-      <c r="F58" s="133"/>
-      <c r="G58" s="134"/>
-      <c r="H58" s="132"/>
-      <c r="I58" s="134"/>
+      <c r="E58" s="149"/>
+      <c r="F58" s="150"/>
+      <c r="G58" s="151"/>
+      <c r="H58" s="149"/>
+      <c r="I58" s="151"/>
     </row>
     <row r="59" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A59" s="135" t="s">
+      <c r="A59" s="143" t="s">
         <v>29</v>
       </c>
-      <c r="B59" s="81"/>
+      <c r="B59" s="101"/>
       <c r="C59" s="35" t="s">
         <v>51</v>
       </c>
       <c r="D59" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="E59" s="136" t="s">
+      <c r="E59" s="152" t="s">
         <v>49</v>
       </c>
-      <c r="F59" s="137"/>
-      <c r="G59" s="138"/>
-      <c r="H59" s="139" t="s">
+      <c r="F59" s="153"/>
+      <c r="G59" s="154"/>
+      <c r="H59" s="155" t="s">
         <v>46</v>
       </c>
-      <c r="I59" s="140"/>
+      <c r="I59" s="156"/>
     </row>
     <row r="60" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A60" s="127" t="s">
+      <c r="A60" s="157" t="s">
         <v>30</v>
       </c>
-      <c r="B60" s="127"/>
+      <c r="B60" s="157"/>
       <c r="C60" s="36"/>
       <c r="D60" s="37"/>
-      <c r="E60" s="128"/>
-      <c r="F60" s="128"/>
-      <c r="G60" s="128"/>
-      <c r="H60" s="129" t="s">
+      <c r="E60" s="158"/>
+      <c r="F60" s="158"/>
+      <c r="G60" s="158"/>
+      <c r="H60" s="159" t="s">
         <v>47</v>
       </c>
-      <c r="I60" s="129"/>
+      <c r="I60" s="159"/>
       <c r="M60" s="38"/>
     </row>
     <row r="61" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A61" s="127" t="s">
+      <c r="A61" s="157" t="s">
         <v>31</v>
       </c>
-      <c r="B61" s="127"/>
+      <c r="B61" s="157"/>
       <c r="C61" s="36"/>
       <c r="D61" s="37"/>
-      <c r="E61" s="128"/>
-      <c r="F61" s="128"/>
-      <c r="G61" s="128"/>
-      <c r="H61" s="129" t="s">
+      <c r="E61" s="158"/>
+      <c r="F61" s="158"/>
+      <c r="G61" s="158"/>
+      <c r="H61" s="159" t="s">
         <v>48</v>
       </c>
-      <c r="I61" s="129"/>
+      <c r="I61" s="159"/>
     </row>
     <row r="62" spans="1:13" ht="13.7" customHeight="1">
+      <c r="A62" t="s">
+        <v>52</v>
+      </c>
       <c r="M62" s="39"/>
     </row>
     <row r="63" spans="1:13" ht="13.7" customHeight="1">
@@ -3470,40 +3543,40 @@
     <row r="17578" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:I1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:I2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:I4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:I6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="C53:D53"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="C50:D50"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="E60:G60"/>
+    <mergeCell ref="H60:I60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="H58:I58"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="B56:I56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="H57:I57"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="C20:D20"/>
@@ -3520,40 +3593,40 @@
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="B55:I55"/>
-    <mergeCell ref="B56:I56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="E57:G57"/>
-    <mergeCell ref="H57:I57"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="E58:G58"/>
-    <mergeCell ref="H58:I58"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="E59:G59"/>
-    <mergeCell ref="H59:I59"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="E60:G60"/>
-    <mergeCell ref="H60:I60"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="H61:I61"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="C53:D53"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:I3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
chore: add tup logo in RIS pdf
</commit_message>
<xml_diff>
--- a/procurement_documents/RIS Template.xlsx
+++ b/procurement_documents/RIS Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0397C4BD-12CE-4064-8D03-40495EDBF07F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38A758F-04CB-4825-8874-F94CF05FB385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,8 +26,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="56">
   <si>
     <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES</t>
   </si>
@@ -189,6 +211,13 @@
   </si>
   <si>
     <t>Scan to receive item/s</t>
+  </si>
+  <si>
+    <t>The Technological University of the Philippines shall be a premiere state university with recognized excellence in engineering and technology education at par with the leading universities in the ASEAN region.</t>
+  </si>
+  <si>
+    <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES
+                          TAGUIG CITY</t>
   </si>
 </sst>
 </file>
@@ -198,7 +227,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="42">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -485,6 +514,14 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -674,7 +711,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="185">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -799,9 +836,6 @@
     <xf numFmtId="43" fontId="32" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -823,197 +857,20 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="28" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="23" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1031,22 +888,259 @@
     <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="28" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="23" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1064,101 +1158,80 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1175,6 +1248,70 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1477,146 +1614,142 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1">
-      <c r="A1" s="58"/>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="164"/>
-      <c r="F1" s="165"/>
-      <c r="G1" s="165"/>
-      <c r="H1" s="165"/>
-      <c r="I1" s="166"/>
+      <c r="A1" s="172" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="B1" s="173"/>
+      <c r="C1" s="181" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="182"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="120"/>
+      <c r="G1" s="120"/>
+      <c r="H1" s="120"/>
+      <c r="I1" s="121"/>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A2" s="64" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="167"/>
-      <c r="F2" s="168"/>
-      <c r="G2" s="168"/>
-      <c r="H2" s="168"/>
-      <c r="I2" s="169"/>
+      <c r="A2" s="122"/>
+      <c r="B2" s="174"/>
+      <c r="C2" s="183"/>
+      <c r="D2" s="184"/>
+      <c r="E2" s="125"/>
+      <c r="F2" s="126"/>
+      <c r="G2" s="126"/>
+      <c r="H2" s="126"/>
+      <c r="I2" s="127"/>
     </row>
     <row r="3" spans="1:9" ht="17.25" customHeight="1">
-      <c r="A3" s="64" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="65"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="70" t="s">
+      <c r="A3" s="122"/>
+      <c r="B3" s="174"/>
+      <c r="C3" s="183"/>
+      <c r="D3" s="184"/>
+      <c r="E3" s="128" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="71"/>
-      <c r="G3" s="71"/>
-      <c r="H3" s="71"/>
-      <c r="I3" s="72"/>
+      <c r="F3" s="129"/>
+      <c r="G3" s="129"/>
+      <c r="H3" s="129"/>
+      <c r="I3" s="130"/>
     </row>
     <row r="4" spans="1:9" ht="15" customHeight="1">
-      <c r="A4" s="73" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="76" t="s">
+      <c r="A4" s="122"/>
+      <c r="B4" s="174"/>
+      <c r="C4" s="183"/>
+      <c r="D4" s="184"/>
+      <c r="E4" s="107" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="77"/>
-      <c r="G4" s="77"/>
-      <c r="H4" s="77"/>
-      <c r="I4" s="78"/>
+      <c r="F4" s="108"/>
+      <c r="G4" s="108"/>
+      <c r="H4" s="108"/>
+      <c r="I4" s="109"/>
     </row>
     <row r="5" spans="1:9" ht="15" customHeight="1">
-      <c r="A5" s="73" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="74"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="79"/>
-      <c r="F5" s="77"/>
-      <c r="G5" s="77"/>
-      <c r="H5" s="77"/>
-      <c r="I5" s="78"/>
+      <c r="A5" s="175" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="176"/>
+      <c r="C5" s="176"/>
+      <c r="D5" s="177"/>
+      <c r="E5" s="110"/>
+      <c r="F5" s="108"/>
+      <c r="G5" s="108"/>
+      <c r="H5" s="108"/>
+      <c r="I5" s="109"/>
     </row>
     <row r="6" spans="1:9" ht="15" customHeight="1">
-      <c r="A6" s="80" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="81"/>
-      <c r="C6" s="81"/>
-      <c r="D6" s="82"/>
-      <c r="E6" s="83"/>
-      <c r="F6" s="84"/>
-      <c r="G6" s="84"/>
-      <c r="H6" s="84"/>
-      <c r="I6" s="85"/>
+      <c r="A6" s="178"/>
+      <c r="B6" s="179"/>
+      <c r="C6" s="179"/>
+      <c r="D6" s="180"/>
+      <c r="E6" s="113"/>
+      <c r="F6" s="114"/>
+      <c r="G6" s="114"/>
+      <c r="H6" s="114"/>
+      <c r="I6" s="115"/>
     </row>
     <row r="7" spans="1:9" ht="20.100000000000001" customHeight="1">
-      <c r="A7" s="162" t="s">
+      <c r="A7" s="92" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="163"/>
-      <c r="C7" s="122" t="s">
+      <c r="B7" s="93"/>
+      <c r="C7" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="123"/>
-      <c r="E7" s="128"/>
-      <c r="F7" s="129"/>
-      <c r="G7" s="129"/>
-      <c r="H7" s="129"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="68"/>
+      <c r="F7" s="69"/>
+      <c r="G7" s="69"/>
+      <c r="H7" s="69"/>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="87"/>
-      <c r="C8" s="87"/>
-      <c r="D8" s="88"/>
-      <c r="E8" s="124" t="s">
+      <c r="B8" s="94"/>
+      <c r="C8" s="94"/>
+      <c r="D8" s="95"/>
+      <c r="E8" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="125"/>
-      <c r="G8" s="125"/>
-      <c r="H8" s="125"/>
-      <c r="I8" s="51"/>
+      <c r="F8" s="65"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="65"/>
+      <c r="I8" s="50"/>
     </row>
     <row r="9" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A9" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="89"/>
-      <c r="C9" s="89"/>
-      <c r="D9" s="90"/>
-      <c r="E9" s="126" t="s">
+      <c r="B9" s="96"/>
+      <c r="C9" s="96"/>
+      <c r="D9" s="97"/>
+      <c r="E9" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="127"/>
-      <c r="G9" s="91"/>
-      <c r="H9" s="91"/>
-      <c r="I9" s="92"/>
+      <c r="F9" s="67"/>
+      <c r="G9" s="98"/>
+      <c r="H9" s="98"/>
+      <c r="I9" s="99"/>
     </row>
     <row r="10" spans="1:9" ht="20.100000000000001" customHeight="1">
-      <c r="A10" s="93" t="s">
+      <c r="A10" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="94"/>
-      <c r="C10" s="94"/>
-      <c r="D10" s="94"/>
-      <c r="E10" s="95"/>
-      <c r="F10" s="96" t="s">
+      <c r="B10" s="101"/>
+      <c r="C10" s="101"/>
+      <c r="D10" s="101"/>
+      <c r="E10" s="102"/>
+      <c r="F10" s="103" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="97"/>
-      <c r="H10" s="93" t="s">
+      <c r="G10" s="104"/>
+      <c r="H10" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="95"/>
+      <c r="I10" s="102"/>
     </row>
     <row r="11" spans="1:9" ht="45" customHeight="1">
       <c r="A11" s="41" t="s">
@@ -1625,10 +1758,10 @@
       <c r="B11" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="100" t="s">
+      <c r="C11" s="90" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="101"/>
+      <c r="D11" s="91"/>
       <c r="E11" s="42" t="s">
         <v>19</v>
       </c>
@@ -1648,583 +1781,648 @@
     <row r="12" spans="1:9" ht="15" customHeight="1">
       <c r="A12" s="44"/>
       <c r="B12" s="45"/>
-      <c r="C12" s="98"/>
-      <c r="D12" s="99"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="61"/>
       <c r="E12" s="48"/>
       <c r="F12" s="46"/>
       <c r="G12" s="49"/>
-      <c r="H12" s="45"/>
-      <c r="I12" s="50"/>
+      <c r="H12" s="170"/>
+      <c r="I12" s="171"/>
     </row>
     <row r="13" spans="1:9" ht="15" customHeight="1">
       <c r="A13" s="44"/>
       <c r="B13" s="45"/>
-      <c r="C13" s="98"/>
-      <c r="D13" s="99"/>
+      <c r="C13" s="60"/>
+      <c r="D13" s="61"/>
       <c r="E13" s="48"/>
       <c r="F13" s="46"/>
       <c r="G13" s="49"/>
-      <c r="H13" s="45"/>
-      <c r="I13" s="50"/>
+      <c r="H13" s="170"/>
+      <c r="I13" s="171"/>
     </row>
     <row r="14" spans="1:9" ht="15" customHeight="1">
       <c r="A14" s="44"/>
       <c r="B14" s="45"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="99"/>
+      <c r="C14" s="60"/>
+      <c r="D14" s="61"/>
       <c r="E14" s="48"/>
       <c r="F14" s="46"/>
       <c r="G14" s="49"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="50"/>
+      <c r="H14" s="170"/>
+      <c r="I14" s="171"/>
     </row>
     <row r="15" spans="1:9" ht="15" customHeight="1">
       <c r="A15" s="44"/>
       <c r="B15" s="45"/>
-      <c r="C15" s="98"/>
-      <c r="D15" s="99"/>
+      <c r="C15" s="60"/>
+      <c r="D15" s="61"/>
       <c r="E15" s="48"/>
       <c r="F15" s="46"/>
       <c r="G15" s="49"/>
-      <c r="H15" s="45"/>
-      <c r="I15" s="50"/>
+      <c r="H15" s="170"/>
+      <c r="I15" s="171"/>
     </row>
     <row r="16" spans="1:9" ht="15" customHeight="1">
       <c r="A16" s="44"/>
       <c r="B16" s="45"/>
-      <c r="C16" s="98"/>
-      <c r="D16" s="99"/>
+      <c r="C16" s="60"/>
+      <c r="D16" s="61"/>
       <c r="E16" s="48"/>
       <c r="F16" s="46"/>
       <c r="G16" s="49"/>
-      <c r="H16" s="45"/>
-      <c r="I16" s="50"/>
+      <c r="H16" s="170"/>
+      <c r="I16" s="171"/>
     </row>
     <row r="17" spans="1:9" ht="15" customHeight="1">
       <c r="A17" s="44"/>
       <c r="B17" s="45"/>
-      <c r="C17" s="98"/>
-      <c r="D17" s="99"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="61"/>
       <c r="E17" s="48"/>
       <c r="F17" s="46"/>
       <c r="G17" s="49"/>
-      <c r="H17" s="45"/>
-      <c r="I17" s="50"/>
+      <c r="H17" s="170"/>
+      <c r="I17" s="171"/>
     </row>
     <row r="18" spans="1:9" ht="15" customHeight="1">
       <c r="A18" s="44"/>
       <c r="B18" s="45"/>
-      <c r="C18" s="98"/>
-      <c r="D18" s="99"/>
+      <c r="C18" s="60"/>
+      <c r="D18" s="61"/>
       <c r="E18" s="48"/>
       <c r="F18" s="46"/>
       <c r="G18" s="49"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="50"/>
+      <c r="H18" s="170"/>
+      <c r="I18" s="171"/>
     </row>
     <row r="19" spans="1:9" ht="15" customHeight="1">
       <c r="A19" s="44"/>
       <c r="B19" s="45"/>
-      <c r="C19" s="98"/>
-      <c r="D19" s="99"/>
+      <c r="C19" s="60"/>
+      <c r="D19" s="61"/>
       <c r="E19" s="48"/>
       <c r="F19" s="46"/>
       <c r="G19" s="49"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="50"/>
+      <c r="H19" s="170"/>
+      <c r="I19" s="171"/>
     </row>
     <row r="20" spans="1:9" ht="15" customHeight="1">
       <c r="A20" s="44"/>
       <c r="B20" s="45"/>
-      <c r="C20" s="98"/>
-      <c r="D20" s="99"/>
+      <c r="C20" s="60"/>
+      <c r="D20" s="61"/>
       <c r="E20" s="48"/>
       <c r="F20" s="46"/>
       <c r="G20" s="49"/>
-      <c r="H20" s="45"/>
-      <c r="I20" s="50"/>
+      <c r="H20" s="170"/>
+      <c r="I20" s="171"/>
     </row>
     <row r="21" spans="1:9" ht="15" customHeight="1">
       <c r="A21" s="44"/>
       <c r="B21" s="45"/>
-      <c r="C21" s="98"/>
-      <c r="D21" s="99"/>
+      <c r="C21" s="60"/>
+      <c r="D21" s="61"/>
       <c r="E21" s="48"/>
       <c r="F21" s="46"/>
       <c r="G21" s="49"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="50"/>
+      <c r="H21" s="170"/>
+      <c r="I21" s="171"/>
     </row>
     <row r="22" spans="1:9" ht="15" customHeight="1">
       <c r="A22" s="44"/>
       <c r="B22" s="45"/>
-      <c r="C22" s="98"/>
-      <c r="D22" s="99"/>
+      <c r="C22" s="60"/>
+      <c r="D22" s="61"/>
       <c r="E22" s="48"/>
       <c r="F22" s="46"/>
       <c r="G22" s="49"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="50"/>
+      <c r="H22" s="170"/>
+      <c r="I22" s="171"/>
     </row>
     <row r="23" spans="1:9" ht="15" customHeight="1">
       <c r="A23" s="44"/>
       <c r="B23" s="45"/>
-      <c r="C23" s="98"/>
-      <c r="D23" s="99"/>
+      <c r="C23" s="60"/>
+      <c r="D23" s="61"/>
       <c r="E23" s="48"/>
       <c r="F23" s="46"/>
       <c r="G23" s="49"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="50"/>
+      <c r="H23" s="170"/>
+      <c r="I23" s="171"/>
     </row>
     <row r="24" spans="1:9" ht="15" customHeight="1">
       <c r="A24" s="44"/>
       <c r="B24" s="45"/>
-      <c r="C24" s="98"/>
-      <c r="D24" s="99"/>
+      <c r="C24" s="60"/>
+      <c r="D24" s="61"/>
       <c r="E24" s="48"/>
       <c r="F24" s="46"/>
       <c r="G24" s="49"/>
-      <c r="H24" s="45"/>
-      <c r="I24" s="50"/>
+      <c r="H24" s="170"/>
+      <c r="I24" s="171"/>
     </row>
     <row r="25" spans="1:9" ht="15" customHeight="1">
       <c r="A25" s="44"/>
       <c r="B25" s="45"/>
-      <c r="C25" s="98"/>
-      <c r="D25" s="99"/>
+      <c r="C25" s="60"/>
+      <c r="D25" s="61"/>
       <c r="E25" s="48"/>
       <c r="F25" s="46"/>
       <c r="G25" s="49"/>
-      <c r="H25" s="45"/>
-      <c r="I25" s="50"/>
+      <c r="H25" s="170"/>
+      <c r="I25" s="171"/>
     </row>
     <row r="26" spans="1:9" ht="15" customHeight="1">
       <c r="A26" s="44"/>
       <c r="B26" s="45"/>
-      <c r="C26" s="98"/>
-      <c r="D26" s="99"/>
+      <c r="C26" s="60"/>
+      <c r="D26" s="61"/>
       <c r="E26" s="48"/>
       <c r="F26" s="46"/>
       <c r="G26" s="49"/>
-      <c r="H26" s="45"/>
-      <c r="I26" s="50"/>
+      <c r="H26" s="170"/>
+      <c r="I26" s="171"/>
     </row>
     <row r="27" spans="1:9" ht="15" customHeight="1">
       <c r="A27" s="44"/>
       <c r="B27" s="45"/>
-      <c r="C27" s="98"/>
-      <c r="D27" s="99"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="61"/>
       <c r="E27" s="48"/>
       <c r="F27" s="46"/>
       <c r="G27" s="49"/>
-      <c r="H27" s="45"/>
-      <c r="I27" s="50"/>
+      <c r="H27" s="170"/>
+      <c r="I27" s="171"/>
     </row>
     <row r="28" spans="1:9" ht="15" customHeight="1">
       <c r="A28" s="44"/>
       <c r="B28" s="45"/>
-      <c r="C28" s="98"/>
-      <c r="D28" s="99"/>
+      <c r="C28" s="60"/>
+      <c r="D28" s="61"/>
       <c r="E28" s="48"/>
       <c r="F28" s="46"/>
       <c r="G28" s="49"/>
-      <c r="H28" s="45"/>
-      <c r="I28" s="50"/>
+      <c r="H28" s="170"/>
+      <c r="I28" s="171"/>
     </row>
     <row r="29" spans="1:9" ht="15" customHeight="1">
       <c r="A29" s="44"/>
       <c r="B29" s="45"/>
-      <c r="C29" s="98"/>
-      <c r="D29" s="99"/>
+      <c r="C29" s="60"/>
+      <c r="D29" s="61"/>
       <c r="E29" s="48"/>
       <c r="F29" s="46"/>
       <c r="G29" s="49"/>
-      <c r="H29" s="45"/>
-      <c r="I29" s="50"/>
+      <c r="H29" s="170"/>
+      <c r="I29" s="171"/>
     </row>
     <row r="30" spans="1:9" ht="15" customHeight="1">
       <c r="A30" s="44"/>
       <c r="B30" s="45"/>
-      <c r="C30" s="98"/>
-      <c r="D30" s="99"/>
+      <c r="C30" s="60"/>
+      <c r="D30" s="61"/>
       <c r="E30" s="48"/>
       <c r="F30" s="46"/>
       <c r="G30" s="49"/>
-      <c r="H30" s="45"/>
-      <c r="I30" s="50"/>
+      <c r="H30" s="170"/>
+      <c r="I30" s="171"/>
     </row>
     <row r="31" spans="1:9" ht="15" customHeight="1">
       <c r="A31" s="44"/>
       <c r="B31" s="45"/>
-      <c r="C31" s="98"/>
-      <c r="D31" s="99"/>
+      <c r="C31" s="60"/>
+      <c r="D31" s="61"/>
       <c r="E31" s="48"/>
       <c r="F31" s="46"/>
       <c r="G31" s="49"/>
-      <c r="H31" s="45"/>
-      <c r="I31" s="50"/>
+      <c r="H31" s="170"/>
+      <c r="I31" s="171"/>
     </row>
     <row r="32" spans="1:9" ht="15" customHeight="1">
       <c r="A32" s="44"/>
       <c r="B32" s="45"/>
-      <c r="C32" s="98"/>
-      <c r="D32" s="99"/>
+      <c r="C32" s="60"/>
+      <c r="D32" s="61"/>
       <c r="E32" s="48"/>
       <c r="F32" s="46"/>
       <c r="G32" s="49"/>
-      <c r="H32" s="45"/>
-      <c r="I32" s="50"/>
+      <c r="H32" s="170"/>
+      <c r="I32" s="171"/>
     </row>
     <row r="33" spans="1:9" ht="15" customHeight="1">
       <c r="A33" s="44"/>
       <c r="B33" s="45"/>
-      <c r="C33" s="98"/>
-      <c r="D33" s="99"/>
+      <c r="C33" s="60"/>
+      <c r="D33" s="61"/>
       <c r="E33" s="48"/>
       <c r="F33" s="46"/>
       <c r="G33" s="49"/>
-      <c r="H33" s="45"/>
-      <c r="I33" s="50"/>
+      <c r="H33" s="170"/>
+      <c r="I33" s="171"/>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1">
       <c r="A34" s="44"/>
       <c r="B34" s="45"/>
-      <c r="C34" s="98"/>
-      <c r="D34" s="99"/>
+      <c r="C34" s="60"/>
+      <c r="D34" s="61"/>
       <c r="E34" s="48"/>
       <c r="F34" s="46"/>
       <c r="G34" s="49"/>
-      <c r="H34" s="45"/>
-      <c r="I34" s="50"/>
+      <c r="H34" s="170"/>
+      <c r="I34" s="171"/>
     </row>
     <row r="35" spans="1:9" ht="15" customHeight="1">
       <c r="A35" s="44"/>
       <c r="B35" s="45"/>
-      <c r="C35" s="98"/>
-      <c r="D35" s="99"/>
+      <c r="C35" s="60"/>
+      <c r="D35" s="61"/>
       <c r="E35" s="48"/>
       <c r="F35" s="46"/>
       <c r="G35" s="49"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="50"/>
+      <c r="H35" s="170"/>
+      <c r="I35" s="171"/>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1">
       <c r="A36" s="44"/>
       <c r="B36" s="45"/>
-      <c r="C36" s="98"/>
-      <c r="D36" s="99"/>
+      <c r="C36" s="60"/>
+      <c r="D36" s="61"/>
       <c r="E36" s="48"/>
       <c r="F36" s="46"/>
       <c r="G36" s="49"/>
-      <c r="H36" s="45"/>
-      <c r="I36" s="50"/>
+      <c r="H36" s="170"/>
+      <c r="I36" s="171"/>
     </row>
     <row r="37" spans="1:9" ht="15" customHeight="1">
       <c r="A37" s="44"/>
       <c r="B37" s="45"/>
-      <c r="C37" s="98"/>
-      <c r="D37" s="99"/>
+      <c r="C37" s="60"/>
+      <c r="D37" s="61"/>
       <c r="E37" s="48"/>
       <c r="F37" s="46"/>
       <c r="G37" s="49"/>
-      <c r="H37" s="45"/>
-      <c r="I37" s="50"/>
+      <c r="H37" s="170"/>
+      <c r="I37" s="171"/>
     </row>
     <row r="38" spans="1:9" ht="15" customHeight="1">
       <c r="A38" s="44"/>
       <c r="B38" s="45"/>
-      <c r="C38" s="98"/>
-      <c r="D38" s="99"/>
+      <c r="C38" s="60"/>
+      <c r="D38" s="61"/>
       <c r="E38" s="48"/>
       <c r="F38" s="46"/>
       <c r="G38" s="49"/>
-      <c r="H38" s="45"/>
-      <c r="I38" s="50"/>
+      <c r="H38" s="170"/>
+      <c r="I38" s="171"/>
     </row>
     <row r="39" spans="1:9" ht="15" customHeight="1">
       <c r="A39" s="44"/>
       <c r="B39" s="45"/>
-      <c r="C39" s="98"/>
-      <c r="D39" s="99"/>
+      <c r="C39" s="60"/>
+      <c r="D39" s="61"/>
       <c r="E39" s="48"/>
       <c r="F39" s="46"/>
       <c r="G39" s="49"/>
-      <c r="H39" s="45"/>
-      <c r="I39" s="50"/>
+      <c r="H39" s="170"/>
+      <c r="I39" s="171"/>
     </row>
     <row r="40" spans="1:9" ht="15" customHeight="1">
       <c r="A40" s="44"/>
       <c r="B40" s="45"/>
-      <c r="C40" s="98"/>
-      <c r="D40" s="99"/>
+      <c r="C40" s="60"/>
+      <c r="D40" s="61"/>
       <c r="E40" s="48"/>
       <c r="F40" s="46"/>
       <c r="G40" s="49"/>
-      <c r="H40" s="45"/>
-      <c r="I40" s="50"/>
+      <c r="H40" s="170"/>
+      <c r="I40" s="171"/>
     </row>
     <row r="41" spans="1:9" ht="15" customHeight="1">
       <c r="A41" s="44"/>
       <c r="B41" s="45"/>
-      <c r="C41" s="98"/>
-      <c r="D41" s="99"/>
+      <c r="C41" s="60"/>
+      <c r="D41" s="61"/>
       <c r="E41" s="48"/>
       <c r="F41" s="46"/>
       <c r="G41" s="49"/>
-      <c r="H41" s="45"/>
-      <c r="I41" s="50"/>
+      <c r="H41" s="170"/>
+      <c r="I41" s="171"/>
     </row>
     <row r="42" spans="1:9" ht="15" customHeight="1">
       <c r="A42" s="44"/>
       <c r="B42" s="45"/>
-      <c r="C42" s="98"/>
-      <c r="D42" s="99"/>
+      <c r="C42" s="60"/>
+      <c r="D42" s="61"/>
       <c r="E42" s="48"/>
       <c r="F42" s="46"/>
       <c r="G42" s="49"/>
-      <c r="H42" s="45"/>
-      <c r="I42" s="50"/>
+      <c r="H42" s="170"/>
+      <c r="I42" s="171"/>
     </row>
     <row r="43" spans="1:9" ht="15" customHeight="1">
       <c r="A43" s="44"/>
       <c r="B43" s="45"/>
-      <c r="C43" s="98"/>
-      <c r="D43" s="99"/>
+      <c r="C43" s="60"/>
+      <c r="D43" s="61"/>
       <c r="E43" s="48"/>
       <c r="F43" s="46"/>
       <c r="G43" s="49"/>
-      <c r="H43" s="45"/>
-      <c r="I43" s="50"/>
+      <c r="H43" s="170"/>
+      <c r="I43" s="171"/>
     </row>
     <row r="44" spans="1:9" ht="15" customHeight="1">
       <c r="A44" s="44"/>
       <c r="B44" s="45"/>
-      <c r="C44" s="98"/>
-      <c r="D44" s="99"/>
+      <c r="C44" s="60"/>
+      <c r="D44" s="61"/>
       <c r="E44" s="48"/>
       <c r="F44" s="46"/>
       <c r="G44" s="49"/>
-      <c r="H44" s="45"/>
-      <c r="I44" s="50"/>
+      <c r="H44" s="170"/>
+      <c r="I44" s="171"/>
     </row>
     <row r="45" spans="1:9" ht="15" customHeight="1">
       <c r="A45" s="44"/>
       <c r="B45" s="45"/>
-      <c r="C45" s="98"/>
-      <c r="D45" s="99"/>
+      <c r="C45" s="60"/>
+      <c r="D45" s="61"/>
       <c r="E45" s="48"/>
       <c r="F45" s="46"/>
       <c r="G45" s="49"/>
-      <c r="H45" s="45"/>
-      <c r="I45" s="50"/>
+      <c r="H45" s="170"/>
+      <c r="I45" s="171"/>
     </row>
     <row r="46" spans="1:9" ht="15" customHeight="1">
       <c r="A46" s="44"/>
       <c r="B46" s="45"/>
-      <c r="C46" s="98"/>
-      <c r="D46" s="99"/>
+      <c r="C46" s="60"/>
+      <c r="D46" s="61"/>
       <c r="E46" s="48"/>
       <c r="F46" s="46"/>
       <c r="G46" s="49"/>
-      <c r="H46" s="45"/>
-      <c r="I46" s="50"/>
+      <c r="H46" s="170"/>
+      <c r="I46" s="171"/>
     </row>
     <row r="47" spans="1:9" ht="15" customHeight="1">
       <c r="A47" s="44"/>
       <c r="B47" s="45"/>
-      <c r="C47" s="98"/>
-      <c r="D47" s="99"/>
+      <c r="C47" s="60"/>
+      <c r="D47" s="61"/>
       <c r="E47" s="48"/>
       <c r="F47" s="46"/>
       <c r="G47" s="49"/>
-      <c r="H47" s="45"/>
-      <c r="I47" s="50"/>
+      <c r="H47" s="170"/>
+      <c r="I47" s="171"/>
     </row>
     <row r="48" spans="1:9" ht="15" customHeight="1">
       <c r="A48" s="44"/>
       <c r="B48" s="45"/>
-      <c r="C48" s="98"/>
-      <c r="D48" s="99"/>
+      <c r="C48" s="60"/>
+      <c r="D48" s="61"/>
       <c r="E48" s="48"/>
       <c r="F48" s="46"/>
       <c r="G48" s="49"/>
-      <c r="H48" s="45"/>
-      <c r="I48" s="50"/>
+      <c r="H48" s="170"/>
+      <c r="I48" s="171"/>
     </row>
     <row r="49" spans="1:9" ht="15" customHeight="1">
       <c r="A49" s="44"/>
       <c r="B49" s="45"/>
-      <c r="C49" s="98"/>
-      <c r="D49" s="99"/>
+      <c r="C49" s="60"/>
+      <c r="D49" s="61"/>
       <c r="E49" s="48"/>
       <c r="F49" s="46"/>
       <c r="G49" s="49"/>
-      <c r="H49" s="45"/>
-      <c r="I49" s="50"/>
+      <c r="H49" s="170"/>
+      <c r="I49" s="171"/>
     </row>
     <row r="50" spans="1:9" ht="15" customHeight="1">
       <c r="A50" s="44"/>
       <c r="B50" s="45"/>
-      <c r="C50" s="98"/>
-      <c r="D50" s="99"/>
+      <c r="C50" s="60"/>
+      <c r="D50" s="61"/>
       <c r="E50" s="48"/>
       <c r="F50" s="46"/>
       <c r="G50" s="49"/>
-      <c r="H50" s="45"/>
-      <c r="I50" s="50"/>
+      <c r="H50" s="170"/>
+      <c r="I50" s="171"/>
     </row>
     <row r="51" spans="1:9" ht="15" customHeight="1">
       <c r="A51" s="44"/>
       <c r="B51" s="45"/>
-      <c r="C51" s="98"/>
-      <c r="D51" s="99"/>
+      <c r="C51" s="60"/>
+      <c r="D51" s="61"/>
       <c r="E51" s="48"/>
       <c r="F51" s="46"/>
       <c r="G51" s="49"/>
-      <c r="H51" s="45"/>
-      <c r="I51" s="50"/>
+      <c r="H51" s="170"/>
+      <c r="I51" s="171"/>
     </row>
     <row r="52" spans="1:9" ht="15" customHeight="1">
       <c r="A52" s="44"/>
       <c r="B52" s="45"/>
-      <c r="C52" s="98"/>
-      <c r="D52" s="99"/>
+      <c r="C52" s="60"/>
+      <c r="D52" s="61"/>
       <c r="E52" s="48"/>
       <c r="F52" s="46"/>
       <c r="G52" s="49"/>
-      <c r="H52" s="45"/>
-      <c r="I52" s="50"/>
+      <c r="H52" s="170"/>
+      <c r="I52" s="171"/>
     </row>
     <row r="53" spans="1:9" ht="15" customHeight="1">
       <c r="A53" s="44"/>
       <c r="B53" s="45"/>
-      <c r="C53" s="98"/>
-      <c r="D53" s="99"/>
+      <c r="C53" s="60"/>
+      <c r="D53" s="61"/>
       <c r="E53" s="48"/>
       <c r="F53" s="46"/>
       <c r="G53" s="49"/>
-      <c r="H53" s="45"/>
-      <c r="I53" s="50"/>
+      <c r="H53" s="170"/>
+      <c r="I53" s="171"/>
     </row>
     <row r="54" spans="1:9" ht="15" customHeight="1">
       <c r="A54" s="44"/>
       <c r="B54" s="45"/>
-      <c r="C54" s="98"/>
-      <c r="D54" s="99"/>
+      <c r="C54" s="60"/>
+      <c r="D54" s="61"/>
       <c r="E54" s="48"/>
       <c r="F54" s="46"/>
       <c r="G54" s="49"/>
-      <c r="H54" s="45"/>
-      <c r="I54" s="50"/>
+      <c r="H54" s="170"/>
+      <c r="I54" s="171"/>
     </row>
     <row r="55" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A55" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="B55" s="102"/>
-      <c r="C55" s="102"/>
-      <c r="D55" s="102"/>
-      <c r="E55" s="102"/>
-      <c r="F55" s="102"/>
-      <c r="G55" s="102"/>
-      <c r="H55" s="102"/>
-      <c r="I55" s="103"/>
+      <c r="B55" s="83"/>
+      <c r="C55" s="83"/>
+      <c r="D55" s="83"/>
+      <c r="E55" s="83"/>
+      <c r="F55" s="83"/>
+      <c r="G55" s="83"/>
+      <c r="H55" s="83"/>
+      <c r="I55" s="84"/>
     </row>
     <row r="56" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A56" s="32"/>
-      <c r="B56" s="104"/>
-      <c r="C56" s="104"/>
-      <c r="D56" s="104"/>
-      <c r="E56" s="104"/>
-      <c r="F56" s="104"/>
-      <c r="G56" s="104"/>
-      <c r="H56" s="104"/>
-      <c r="I56" s="105"/>
+      <c r="B56" s="85"/>
+      <c r="C56" s="85"/>
+      <c r="D56" s="85"/>
+      <c r="E56" s="85"/>
+      <c r="F56" s="85"/>
+      <c r="G56" s="85"/>
+      <c r="H56" s="85"/>
+      <c r="I56" s="86"/>
     </row>
     <row r="57" spans="1:9" ht="20.100000000000001" customHeight="1">
-      <c r="A57" s="106"/>
-      <c r="B57" s="107"/>
-      <c r="C57" s="53" t="s">
+      <c r="A57" s="87"/>
+      <c r="B57" s="88"/>
+      <c r="C57" s="52" t="s">
         <v>24</v>
       </c>
-      <c r="D57" s="53" t="s">
+      <c r="D57" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="E57" s="108" t="s">
+      <c r="E57" s="75" t="s">
         <v>26</v>
       </c>
-      <c r="F57" s="109"/>
-      <c r="G57" s="110"/>
-      <c r="H57" s="108" t="s">
+      <c r="F57" s="89"/>
+      <c r="G57" s="76"/>
+      <c r="H57" s="75" t="s">
         <v>27</v>
       </c>
-      <c r="I57" s="110"/>
+      <c r="I57" s="76"/>
     </row>
     <row r="58" spans="1:9" ht="20.100000000000001" customHeight="1">
-      <c r="A58" s="108" t="s">
+      <c r="A58" s="75" t="s">
         <v>28</v>
       </c>
-      <c r="B58" s="110"/>
-      <c r="C58" s="54"/>
-      <c r="D58" s="54"/>
-      <c r="E58" s="111"/>
-      <c r="F58" s="112"/>
-      <c r="G58" s="113"/>
-      <c r="H58" s="111"/>
-      <c r="I58" s="113"/>
+      <c r="B58" s="76"/>
+      <c r="C58" s="53"/>
+      <c r="D58" s="53"/>
+      <c r="E58" s="77"/>
+      <c r="F58" s="78"/>
+      <c r="G58" s="79"/>
+      <c r="H58" s="77"/>
+      <c r="I58" s="79"/>
     </row>
     <row r="59" spans="1:9" ht="20.100000000000001" customHeight="1">
-      <c r="A59" s="108" t="s">
+      <c r="A59" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="B59" s="110"/>
-      <c r="C59" s="56"/>
-      <c r="D59" s="57"/>
-      <c r="E59" s="114"/>
-      <c r="F59" s="115"/>
-      <c r="G59" s="116"/>
-      <c r="H59" s="114"/>
-      <c r="I59" s="116"/>
+      <c r="B59" s="76"/>
+      <c r="C59" s="55"/>
+      <c r="D59" s="56"/>
+      <c r="E59" s="80"/>
+      <c r="F59" s="81"/>
+      <c r="G59" s="82"/>
+      <c r="H59" s="80"/>
+      <c r="I59" s="82"/>
     </row>
     <row r="60" spans="1:9" ht="20.100000000000001" customHeight="1">
-      <c r="A60" s="117" t="s">
+      <c r="A60" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="B60" s="117"/>
-      <c r="C60" s="55"/>
-      <c r="D60" s="55"/>
-      <c r="E60" s="118"/>
-      <c r="F60" s="118"/>
-      <c r="G60" s="118"/>
-      <c r="H60" s="119"/>
-      <c r="I60" s="119"/>
+      <c r="B60" s="70"/>
+      <c r="C60" s="54"/>
+      <c r="D60" s="54"/>
+      <c r="E60" s="71"/>
+      <c r="F60" s="71"/>
+      <c r="G60" s="71"/>
+      <c r="H60" s="72"/>
+      <c r="I60" s="72"/>
     </row>
     <row r="61" spans="1:9" ht="20.100000000000001" customHeight="1">
-      <c r="A61" s="117" t="s">
+      <c r="A61" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="B61" s="117"/>
-      <c r="C61" s="52"/>
-      <c r="D61" s="52"/>
-      <c r="E61" s="120"/>
-      <c r="F61" s="120"/>
-      <c r="G61" s="120"/>
-      <c r="H61" s="121"/>
-      <c r="I61" s="121"/>
+      <c r="B61" s="70"/>
+      <c r="C61" s="51"/>
+      <c r="D61" s="51"/>
+      <c r="E61" s="73"/>
+      <c r="F61" s="73"/>
+      <c r="G61" s="73"/>
+      <c r="H61" s="74"/>
+      <c r="I61" s="74"/>
     </row>
     <row r="62" spans="1:9">
-      <c r="A62" s="171"/>
-      <c r="B62" s="172" t="s">
+      <c r="A62" s="58"/>
+      <c r="B62" s="59" t="s">
         <v>53</v>
       </c>
-      <c r="C62" s="170"/>
+      <c r="C62" s="57"/>
     </row>
     <row r="63" spans="1:9" ht="15" customHeight="1">
-      <c r="C63" s="170"/>
+      <c r="C63" s="57"/>
     </row>
   </sheetData>
-  <mergeCells count="84">
+  <mergeCells count="81">
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="A1:B4"/>
+    <mergeCell ref="C1:D4"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="A5:D6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="B56:I56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="H57:I57"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="H58:I58"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="E60:G60"/>
+    <mergeCell ref="H60:I60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="H61:I61"/>
     <mergeCell ref="C51:D51"/>
     <mergeCell ref="C52:D52"/>
     <mergeCell ref="C53:D53"/>
@@ -2241,74 +2439,6 @@
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="C39:D39"/>
     <mergeCell ref="C40:D40"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="E60:G60"/>
-    <mergeCell ref="H60:I60"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="H61:I61"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="E58:G58"/>
-    <mergeCell ref="H58:I58"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="E59:G59"/>
-    <mergeCell ref="H59:I59"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="B55:I55"/>
-    <mergeCell ref="B56:I56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="E57:G57"/>
-    <mergeCell ref="H57:I57"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:I4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:I6"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:I1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:I2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:I3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -2331,117 +2461,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="58"/>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="63"/>
+      <c r="A1" s="116"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="118"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="163"/>
+      <c r="G1" s="163"/>
+      <c r="H1" s="163"/>
+      <c r="I1" s="164"/>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A2" s="130" t="s">
+      <c r="A2" s="165" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="69"/>
+      <c r="B2" s="123"/>
+      <c r="C2" s="123"/>
+      <c r="D2" s="124"/>
+      <c r="E2" s="166"/>
+      <c r="F2" s="167"/>
+      <c r="G2" s="167"/>
+      <c r="H2" s="167"/>
+      <c r="I2" s="168"/>
     </row>
     <row r="3" spans="1:9" ht="17.25" customHeight="1">
-      <c r="A3" s="130" t="s">
+      <c r="A3" s="165" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="65"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="131" t="s">
+      <c r="B3" s="123"/>
+      <c r="C3" s="123"/>
+      <c r="D3" s="124"/>
+      <c r="E3" s="169" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="71"/>
-      <c r="G3" s="71"/>
-      <c r="H3" s="71"/>
-      <c r="I3" s="72"/>
+      <c r="F3" s="129"/>
+      <c r="G3" s="129"/>
+      <c r="H3" s="129"/>
+      <c r="I3" s="130"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="132" t="s">
+      <c r="A4" s="160" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="79" t="s">
+      <c r="B4" s="105"/>
+      <c r="C4" s="105"/>
+      <c r="D4" s="106"/>
+      <c r="E4" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="77"/>
-      <c r="G4" s="77"/>
-      <c r="H4" s="77"/>
-      <c r="I4" s="78"/>
+      <c r="F4" s="108"/>
+      <c r="G4" s="108"/>
+      <c r="H4" s="108"/>
+      <c r="I4" s="109"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="132" t="s">
+      <c r="A5" s="160" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="74"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="79"/>
-      <c r="F5" s="77"/>
-      <c r="G5" s="77"/>
-      <c r="H5" s="77"/>
-      <c r="I5" s="78"/>
+      <c r="B5" s="105"/>
+      <c r="C5" s="105"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="110"/>
+      <c r="F5" s="108"/>
+      <c r="G5" s="108"/>
+      <c r="H5" s="108"/>
+      <c r="I5" s="109"/>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="133" t="s">
+      <c r="A6" s="161" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="81"/>
-      <c r="C6" s="81"/>
-      <c r="D6" s="82"/>
-      <c r="E6" s="83"/>
-      <c r="F6" s="84"/>
-      <c r="G6" s="84"/>
-      <c r="H6" s="84"/>
-      <c r="I6" s="85"/>
+      <c r="B6" s="111"/>
+      <c r="C6" s="111"/>
+      <c r="D6" s="112"/>
+      <c r="E6" s="113"/>
+      <c r="F6" s="114"/>
+      <c r="G6" s="114"/>
+      <c r="H6" s="114"/>
+      <c r="I6" s="115"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="134" t="s">
+      <c r="A7" s="152" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="86"/>
-      <c r="C7" s="160" t="s">
+      <c r="B7" s="153"/>
+      <c r="C7" s="133" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="161" t="s">
+      <c r="D7" s="134" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="128"/>
-      <c r="F7" s="129"/>
-      <c r="G7" s="129"/>
-      <c r="H7" s="129"/>
+      <c r="E7" s="68"/>
+      <c r="F7" s="69"/>
+      <c r="G7" s="69"/>
+      <c r="H7" s="69"/>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="135" t="s">
+      <c r="B8" s="154" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="135"/>
-      <c r="D8" s="136"/>
-      <c r="E8" s="128" t="s">
+      <c r="C8" s="154"/>
+      <c r="D8" s="155"/>
+      <c r="E8" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="129"/>
-      <c r="G8" s="129"/>
-      <c r="H8" s="129"/>
+      <c r="F8" s="69"/>
+      <c r="G8" s="69"/>
+      <c r="H8" s="69"/>
       <c r="I8" s="3" t="s">
         <v>34</v>
       </c>
@@ -2450,37 +2580,37 @@
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="135" t="s">
+      <c r="B9" s="154" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="135"/>
-      <c r="D9" s="136"/>
-      <c r="E9" s="128" t="s">
+      <c r="C9" s="154"/>
+      <c r="D9" s="155"/>
+      <c r="E9" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="129"/>
-      <c r="G9" s="137" t="s">
+      <c r="F9" s="69"/>
+      <c r="G9" s="156" t="s">
         <v>36</v>
       </c>
-      <c r="H9" s="137"/>
-      <c r="I9" s="138"/>
+      <c r="H9" s="156"/>
+      <c r="I9" s="157"/>
     </row>
     <row r="10" spans="1:9" ht="15" customHeight="1">
-      <c r="A10" s="139" t="s">
+      <c r="A10" s="158" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="94"/>
-      <c r="C10" s="94"/>
-      <c r="D10" s="94"/>
-      <c r="E10" s="95"/>
-      <c r="F10" s="140" t="s">
+      <c r="B10" s="101"/>
+      <c r="C10" s="101"/>
+      <c r="D10" s="101"/>
+      <c r="E10" s="102"/>
+      <c r="F10" s="159" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="97"/>
-      <c r="H10" s="139" t="s">
+      <c r="G10" s="104"/>
+      <c r="H10" s="158" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="95"/>
+      <c r="I10" s="102"/>
     </row>
     <row r="11" spans="1:9" ht="30" customHeight="1">
       <c r="A11" s="4" t="s">
@@ -2492,7 +2622,7 @@
       <c r="C11" s="143" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="101"/>
+      <c r="D11" s="91"/>
       <c r="E11" s="5" t="s">
         <v>19</v>
       </c>
@@ -2516,10 +2646,10 @@
       <c r="B12" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="141" t="s">
+      <c r="C12" s="131" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="142"/>
+      <c r="D12" s="132"/>
       <c r="E12" s="7" t="s">
         <v>40</v>
       </c>
@@ -2539,8 +2669,8 @@
     <row r="13" spans="1:9" ht="13.7" customHeight="1">
       <c r="A13" s="4"/>
       <c r="B13" s="6"/>
-      <c r="C13" s="141"/>
-      <c r="D13" s="142"/>
+      <c r="C13" s="131"/>
+      <c r="D13" s="132"/>
       <c r="E13" s="11"/>
       <c r="F13" s="8"/>
       <c r="G13" s="9"/>
@@ -2550,8 +2680,8 @@
     <row r="14" spans="1:9" ht="13.7" customHeight="1">
       <c r="A14" s="4"/>
       <c r="B14" s="6"/>
-      <c r="C14" s="141"/>
-      <c r="D14" s="142"/>
+      <c r="C14" s="131"/>
+      <c r="D14" s="132"/>
       <c r="E14" s="11"/>
       <c r="F14" s="8"/>
       <c r="G14" s="9"/>
@@ -2561,8 +2691,8 @@
     <row r="15" spans="1:9" ht="13.7" customHeight="1">
       <c r="A15" s="4"/>
       <c r="B15" s="6"/>
-      <c r="C15" s="141"/>
-      <c r="D15" s="142"/>
+      <c r="C15" s="131"/>
+      <c r="D15" s="132"/>
       <c r="E15" s="13"/>
       <c r="F15" s="8"/>
       <c r="G15" s="9"/>
@@ -2572,8 +2702,8 @@
     <row r="16" spans="1:9" ht="13.7" customHeight="1">
       <c r="A16" s="4"/>
       <c r="B16" s="6"/>
-      <c r="C16" s="141"/>
-      <c r="D16" s="142"/>
+      <c r="C16" s="131"/>
+      <c r="D16" s="132"/>
       <c r="E16" s="13"/>
       <c r="F16" s="8"/>
       <c r="G16" s="9"/>
@@ -2583,8 +2713,8 @@
     <row r="17" spans="1:9" ht="13.7" customHeight="1">
       <c r="A17" s="4"/>
       <c r="B17" s="6"/>
-      <c r="C17" s="141"/>
-      <c r="D17" s="142"/>
+      <c r="C17" s="131"/>
+      <c r="D17" s="132"/>
       <c r="E17" s="13"/>
       <c r="F17" s="8"/>
       <c r="G17" s="9"/>
@@ -2594,8 +2724,8 @@
     <row r="18" spans="1:9" ht="13.7" customHeight="1">
       <c r="A18" s="4"/>
       <c r="B18" s="6"/>
-      <c r="C18" s="141"/>
-      <c r="D18" s="142"/>
+      <c r="C18" s="131"/>
+      <c r="D18" s="132"/>
       <c r="E18" s="13"/>
       <c r="F18" s="8"/>
       <c r="G18" s="9"/>
@@ -2605,8 +2735,8 @@
     <row r="19" spans="1:9" ht="13.7" customHeight="1">
       <c r="A19" s="15"/>
       <c r="B19" s="6"/>
-      <c r="C19" s="141"/>
-      <c r="D19" s="142"/>
+      <c r="C19" s="131"/>
+      <c r="D19" s="132"/>
       <c r="E19" s="16"/>
       <c r="F19" s="8"/>
       <c r="G19" s="9"/>
@@ -2616,8 +2746,8 @@
     <row r="20" spans="1:9" ht="13.7" customHeight="1">
       <c r="A20" s="15"/>
       <c r="B20" s="6"/>
-      <c r="C20" s="141"/>
-      <c r="D20" s="142"/>
+      <c r="C20" s="131"/>
+      <c r="D20" s="132"/>
       <c r="E20" s="16"/>
       <c r="F20" s="8"/>
       <c r="G20" s="9"/>
@@ -2627,8 +2757,8 @@
     <row r="21" spans="1:9" ht="13.7" customHeight="1">
       <c r="A21" s="15"/>
       <c r="B21" s="6"/>
-      <c r="C21" s="141"/>
-      <c r="D21" s="142"/>
+      <c r="C21" s="131"/>
+      <c r="D21" s="132"/>
       <c r="E21" s="16"/>
       <c r="F21" s="8"/>
       <c r="G21" s="9"/>
@@ -2638,8 +2768,8 @@
     <row r="22" spans="1:9" ht="13.7" customHeight="1">
       <c r="A22" s="18"/>
       <c r="B22" s="6"/>
-      <c r="C22" s="141"/>
-      <c r="D22" s="142"/>
+      <c r="C22" s="131"/>
+      <c r="D22" s="132"/>
       <c r="E22" s="19"/>
       <c r="F22" s="20"/>
       <c r="G22" s="21"/>
@@ -2649,8 +2779,8 @@
     <row r="23" spans="1:9" ht="13.7" customHeight="1">
       <c r="A23" s="18"/>
       <c r="B23" s="6"/>
-      <c r="C23" s="141"/>
-      <c r="D23" s="142"/>
+      <c r="C23" s="131"/>
+      <c r="D23" s="132"/>
       <c r="E23" s="19"/>
       <c r="F23" s="22"/>
       <c r="G23" s="21"/>
@@ -2660,8 +2790,8 @@
     <row r="24" spans="1:9" ht="13.7" customHeight="1">
       <c r="A24" s="18"/>
       <c r="B24" s="6"/>
-      <c r="C24" s="141"/>
-      <c r="D24" s="142"/>
+      <c r="C24" s="131"/>
+      <c r="D24" s="132"/>
       <c r="E24" s="19"/>
       <c r="F24" s="22"/>
       <c r="G24" s="21"/>
@@ -2671,8 +2801,8 @@
     <row r="25" spans="1:9" ht="13.7" customHeight="1">
       <c r="A25" s="18"/>
       <c r="B25" s="6"/>
-      <c r="C25" s="141"/>
-      <c r="D25" s="142"/>
+      <c r="C25" s="131"/>
+      <c r="D25" s="132"/>
       <c r="E25" s="19"/>
       <c r="F25" s="22"/>
       <c r="G25" s="21"/>
@@ -2682,8 +2812,8 @@
     <row r="26" spans="1:9" ht="13.7" customHeight="1">
       <c r="A26" s="18"/>
       <c r="B26" s="6"/>
-      <c r="C26" s="141"/>
-      <c r="D26" s="142"/>
+      <c r="C26" s="131"/>
+      <c r="D26" s="132"/>
       <c r="E26" s="19"/>
       <c r="F26" s="22"/>
       <c r="G26" s="21"/>
@@ -2693,8 +2823,8 @@
     <row r="27" spans="1:9" ht="13.7" customHeight="1">
       <c r="A27" s="18"/>
       <c r="B27" s="6"/>
-      <c r="C27" s="141"/>
-      <c r="D27" s="142"/>
+      <c r="C27" s="131"/>
+      <c r="D27" s="132"/>
       <c r="E27" s="19"/>
       <c r="F27" s="22"/>
       <c r="G27" s="21"/>
@@ -2704,8 +2834,8 @@
     <row r="28" spans="1:9" ht="13.7" customHeight="1">
       <c r="A28" s="18"/>
       <c r="B28" s="6"/>
-      <c r="C28" s="141"/>
-      <c r="D28" s="142"/>
+      <c r="C28" s="131"/>
+      <c r="D28" s="132"/>
       <c r="E28" s="19"/>
       <c r="F28" s="22"/>
       <c r="G28" s="21"/>
@@ -2715,8 +2845,8 @@
     <row r="29" spans="1:9" ht="13.7" customHeight="1">
       <c r="A29" s="15"/>
       <c r="B29" s="6"/>
-      <c r="C29" s="141"/>
-      <c r="D29" s="142"/>
+      <c r="C29" s="131"/>
+      <c r="D29" s="132"/>
       <c r="E29" s="19"/>
       <c r="F29" s="8"/>
       <c r="G29" s="9"/>
@@ -2726,8 +2856,8 @@
     <row r="30" spans="1:9" ht="13.7" customHeight="1">
       <c r="A30" s="15"/>
       <c r="B30" s="6"/>
-      <c r="C30" s="141"/>
-      <c r="D30" s="142"/>
+      <c r="C30" s="131"/>
+      <c r="D30" s="132"/>
       <c r="E30" s="19"/>
       <c r="F30" s="8"/>
       <c r="G30" s="9"/>
@@ -2737,8 +2867,8 @@
     <row r="31" spans="1:9" ht="13.7" customHeight="1">
       <c r="A31" s="15"/>
       <c r="B31" s="6"/>
-      <c r="C31" s="141"/>
-      <c r="D31" s="142"/>
+      <c r="C31" s="131"/>
+      <c r="D31" s="132"/>
       <c r="E31" s="19"/>
       <c r="F31" s="8"/>
       <c r="G31" s="9"/>
@@ -2748,8 +2878,8 @@
     <row r="32" spans="1:9" ht="13.7" customHeight="1">
       <c r="A32" s="15"/>
       <c r="B32" s="6"/>
-      <c r="C32" s="141"/>
-      <c r="D32" s="142"/>
+      <c r="C32" s="131"/>
+      <c r="D32" s="132"/>
       <c r="E32" s="19"/>
       <c r="F32" s="8"/>
       <c r="G32" s="9"/>
@@ -2759,8 +2889,8 @@
     <row r="33" spans="1:15" ht="13.7" customHeight="1">
       <c r="A33" s="15"/>
       <c r="B33" s="6"/>
-      <c r="C33" s="141"/>
-      <c r="D33" s="142"/>
+      <c r="C33" s="131"/>
+      <c r="D33" s="132"/>
       <c r="E33" s="19"/>
       <c r="F33" s="25"/>
       <c r="G33" s="9"/>
@@ -2770,8 +2900,8 @@
     <row r="34" spans="1:15" ht="13.7" customHeight="1">
       <c r="A34" s="15"/>
       <c r="B34" s="6"/>
-      <c r="C34" s="141"/>
-      <c r="D34" s="142"/>
+      <c r="C34" s="131"/>
+      <c r="D34" s="132"/>
       <c r="E34" s="19"/>
       <c r="F34" s="26"/>
       <c r="G34" s="9"/>
@@ -2781,8 +2911,8 @@
     <row r="35" spans="1:15" ht="13.7" customHeight="1">
       <c r="A35" s="15"/>
       <c r="B35" s="6"/>
-      <c r="C35" s="141"/>
-      <c r="D35" s="142"/>
+      <c r="C35" s="131"/>
+      <c r="D35" s="132"/>
       <c r="E35" s="19"/>
       <c r="F35" s="26"/>
       <c r="G35" s="9"/>
@@ -2792,8 +2922,8 @@
     <row r="36" spans="1:15" ht="13.7" customHeight="1">
       <c r="A36" s="15"/>
       <c r="B36" s="6"/>
-      <c r="C36" s="141"/>
-      <c r="D36" s="142"/>
+      <c r="C36" s="131"/>
+      <c r="D36" s="132"/>
       <c r="E36" s="19"/>
       <c r="F36" s="26"/>
       <c r="G36" s="9"/>
@@ -2803,8 +2933,8 @@
     <row r="37" spans="1:15" ht="13.7" customHeight="1">
       <c r="A37" s="15"/>
       <c r="B37" s="27"/>
-      <c r="C37" s="141"/>
-      <c r="D37" s="142"/>
+      <c r="C37" s="131"/>
+      <c r="D37" s="132"/>
       <c r="E37" s="19"/>
       <c r="F37" s="26"/>
       <c r="G37" s="9"/>
@@ -2814,8 +2944,8 @@
     <row r="38" spans="1:15" ht="13.7" customHeight="1">
       <c r="A38" s="15"/>
       <c r="B38" s="6"/>
-      <c r="C38" s="141"/>
-      <c r="D38" s="142"/>
+      <c r="C38" s="131"/>
+      <c r="D38" s="132"/>
       <c r="E38" s="7"/>
       <c r="F38" s="26"/>
       <c r="G38" s="9"/>
@@ -2828,8 +2958,8 @@
     <row r="39" spans="1:15" ht="13.7" customHeight="1">
       <c r="A39" s="15"/>
       <c r="B39" s="6"/>
-      <c r="C39" s="141"/>
-      <c r="D39" s="142"/>
+      <c r="C39" s="131"/>
+      <c r="D39" s="132"/>
       <c r="E39" s="28"/>
       <c r="F39" s="26"/>
       <c r="G39" s="9"/>
@@ -2839,8 +2969,8 @@
     <row r="40" spans="1:15" ht="13.7" customHeight="1">
       <c r="A40" s="15"/>
       <c r="B40" s="6"/>
-      <c r="C40" s="141"/>
-      <c r="D40" s="142"/>
+      <c r="C40" s="131"/>
+      <c r="D40" s="132"/>
       <c r="E40" s="28"/>
       <c r="F40" s="26"/>
       <c r="G40" s="9"/>
@@ -2850,8 +2980,8 @@
     <row r="41" spans="1:15" ht="13.7" customHeight="1">
       <c r="A41" s="15"/>
       <c r="B41" s="6"/>
-      <c r="C41" s="141"/>
-      <c r="D41" s="142"/>
+      <c r="C41" s="131"/>
+      <c r="D41" s="132"/>
       <c r="E41" s="28"/>
       <c r="F41" s="26"/>
       <c r="G41" s="9"/>
@@ -2861,8 +2991,8 @@
     <row r="42" spans="1:15" ht="13.7" customHeight="1">
       <c r="A42" s="15"/>
       <c r="B42" s="6"/>
-      <c r="C42" s="141"/>
-      <c r="D42" s="142"/>
+      <c r="C42" s="131"/>
+      <c r="D42" s="132"/>
       <c r="E42" s="28"/>
       <c r="F42" s="26"/>
       <c r="G42" s="9"/>
@@ -2872,8 +3002,8 @@
     <row r="43" spans="1:15" ht="13.7" customHeight="1">
       <c r="A43" s="15"/>
       <c r="B43" s="6"/>
-      <c r="C43" s="141"/>
-      <c r="D43" s="142"/>
+      <c r="C43" s="131"/>
+      <c r="D43" s="132"/>
       <c r="E43" s="28"/>
       <c r="F43" s="26"/>
       <c r="G43" s="9"/>
@@ -2886,8 +3016,8 @@
     <row r="44" spans="1:15" ht="13.7" customHeight="1">
       <c r="A44" s="15"/>
       <c r="B44" s="6"/>
-      <c r="C44" s="141"/>
-      <c r="D44" s="142"/>
+      <c r="C44" s="131"/>
+      <c r="D44" s="132"/>
       <c r="E44" s="28"/>
       <c r="F44" s="26"/>
       <c r="G44" s="9"/>
@@ -2897,8 +3027,8 @@
     <row r="45" spans="1:15" ht="13.7" customHeight="1">
       <c r="A45" s="15"/>
       <c r="B45" s="6"/>
-      <c r="C45" s="141"/>
-      <c r="D45" s="142"/>
+      <c r="C45" s="131"/>
+      <c r="D45" s="132"/>
       <c r="E45" s="28"/>
       <c r="F45" s="26"/>
       <c r="G45" s="9"/>
@@ -2908,8 +3038,8 @@
     <row r="46" spans="1:15" ht="13.7" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="6"/>
-      <c r="C46" s="141"/>
-      <c r="D46" s="142"/>
+      <c r="C46" s="131"/>
+      <c r="D46" s="132"/>
       <c r="E46" s="8"/>
       <c r="F46" s="26"/>
       <c r="G46" s="9"/>
@@ -2919,8 +3049,8 @@
     <row r="47" spans="1:15" ht="13.7" customHeight="1">
       <c r="A47" s="15"/>
       <c r="B47" s="6"/>
-      <c r="C47" s="141"/>
-      <c r="D47" s="142"/>
+      <c r="C47" s="131"/>
+      <c r="D47" s="132"/>
       <c r="E47" s="28"/>
       <c r="F47" s="26"/>
       <c r="G47" s="9"/>
@@ -2930,8 +3060,8 @@
     <row r="48" spans="1:15" ht="13.7" customHeight="1">
       <c r="A48" s="15"/>
       <c r="B48" s="6"/>
-      <c r="C48" s="141"/>
-      <c r="D48" s="142"/>
+      <c r="C48" s="131"/>
+      <c r="D48" s="132"/>
       <c r="E48" s="28"/>
       <c r="F48" s="26"/>
       <c r="G48" s="9"/>
@@ -2941,8 +3071,8 @@
     <row r="49" spans="1:13" ht="13.7" customHeight="1">
       <c r="A49" s="15"/>
       <c r="B49" s="29"/>
-      <c r="C49" s="141"/>
-      <c r="D49" s="142"/>
+      <c r="C49" s="131"/>
+      <c r="D49" s="132"/>
       <c r="E49" s="28"/>
       <c r="F49" s="26"/>
       <c r="G49" s="9"/>
@@ -2952,8 +3082,8 @@
     <row r="50" spans="1:13" ht="13.7" hidden="1" customHeight="1">
       <c r="A50" s="15"/>
       <c r="B50" s="6"/>
-      <c r="C50" s="141"/>
-      <c r="D50" s="142"/>
+      <c r="C50" s="131"/>
+      <c r="D50" s="132"/>
       <c r="E50" s="28"/>
       <c r="F50" s="26"/>
       <c r="G50" s="9"/>
@@ -2963,8 +3093,8 @@
     <row r="51" spans="1:13" ht="13.7" customHeight="1">
       <c r="A51" s="15"/>
       <c r="B51" s="6"/>
-      <c r="C51" s="141"/>
-      <c r="D51" s="142"/>
+      <c r="C51" s="131"/>
+      <c r="D51" s="132"/>
       <c r="E51" s="28"/>
       <c r="F51" s="26"/>
       <c r="G51" s="9"/>
@@ -2974,8 +3104,8 @@
     <row r="52" spans="1:13" ht="13.7" customHeight="1">
       <c r="A52" s="15"/>
       <c r="B52" s="29"/>
-      <c r="C52" s="141"/>
-      <c r="D52" s="142"/>
+      <c r="C52" s="131"/>
+      <c r="D52" s="132"/>
       <c r="E52" s="28"/>
       <c r="F52" s="26"/>
       <c r="G52" s="9"/>
@@ -2985,8 +3115,8 @@
     <row r="53" spans="1:13" ht="13.7" customHeight="1">
       <c r="A53" s="15"/>
       <c r="B53" s="6"/>
-      <c r="C53" s="141"/>
-      <c r="D53" s="142"/>
+      <c r="C53" s="131"/>
+      <c r="D53" s="132"/>
       <c r="E53" s="28"/>
       <c r="F53" s="26"/>
       <c r="G53" s="9"/>
@@ -2996,8 +3126,8 @@
     <row r="54" spans="1:13" ht="13.7" customHeight="1">
       <c r="A54" s="15"/>
       <c r="B54" s="29"/>
-      <c r="C54" s="141"/>
-      <c r="D54" s="142"/>
+      <c r="C54" s="131"/>
+      <c r="D54" s="132"/>
       <c r="E54" s="28"/>
       <c r="F54" s="26"/>
       <c r="G54" s="9"/>
@@ -3008,111 +3138,111 @@
       <c r="A55" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="B55" s="144" t="s">
+      <c r="B55" s="149" t="s">
         <v>45</v>
       </c>
-      <c r="C55" s="144"/>
-      <c r="D55" s="144"/>
-      <c r="E55" s="144"/>
-      <c r="F55" s="144"/>
-      <c r="G55" s="144"/>
-      <c r="H55" s="144"/>
-      <c r="I55" s="145"/>
+      <c r="C55" s="149"/>
+      <c r="D55" s="149"/>
+      <c r="E55" s="149"/>
+      <c r="F55" s="149"/>
+      <c r="G55" s="149"/>
+      <c r="H55" s="149"/>
+      <c r="I55" s="150"/>
     </row>
     <row r="56" spans="1:13" ht="13.7" customHeight="1">
       <c r="A56" s="32"/>
-      <c r="B56" s="104"/>
-      <c r="C56" s="104"/>
-      <c r="D56" s="104"/>
-      <c r="E56" s="104"/>
-      <c r="F56" s="104"/>
-      <c r="G56" s="104"/>
-      <c r="H56" s="104"/>
-      <c r="I56" s="105"/>
+      <c r="B56" s="85"/>
+      <c r="C56" s="85"/>
+      <c r="D56" s="85"/>
+      <c r="E56" s="85"/>
+      <c r="F56" s="85"/>
+      <c r="G56" s="85"/>
+      <c r="H56" s="85"/>
+      <c r="I56" s="86"/>
     </row>
     <row r="57" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A57" s="146"/>
-      <c r="B57" s="147"/>
+      <c r="A57" s="138"/>
+      <c r="B57" s="139"/>
       <c r="C57" s="33" t="s">
         <v>24</v>
       </c>
       <c r="D57" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="E57" s="146" t="s">
+      <c r="E57" s="138" t="s">
         <v>26</v>
       </c>
-      <c r="F57" s="148"/>
-      <c r="G57" s="147"/>
-      <c r="H57" s="146" t="s">
+      <c r="F57" s="151"/>
+      <c r="G57" s="139"/>
+      <c r="H57" s="138" t="s">
         <v>27</v>
       </c>
-      <c r="I57" s="147"/>
+      <c r="I57" s="139"/>
     </row>
     <row r="58" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A58" s="146" t="s">
+      <c r="A58" s="138" t="s">
         <v>28</v>
       </c>
-      <c r="B58" s="147"/>
+      <c r="B58" s="139"/>
       <c r="C58" s="34"/>
       <c r="D58" s="34"/>
-      <c r="E58" s="149"/>
-      <c r="F58" s="150"/>
-      <c r="G58" s="151"/>
-      <c r="H58" s="149"/>
-      <c r="I58" s="151"/>
+      <c r="E58" s="140"/>
+      <c r="F58" s="141"/>
+      <c r="G58" s="142"/>
+      <c r="H58" s="140"/>
+      <c r="I58" s="142"/>
     </row>
     <row r="59" spans="1:13" ht="13.7" customHeight="1">
       <c r="A59" s="143" t="s">
         <v>29</v>
       </c>
-      <c r="B59" s="101"/>
+      <c r="B59" s="91"/>
       <c r="C59" s="35" t="s">
         <v>51</v>
       </c>
       <c r="D59" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="E59" s="152" t="s">
+      <c r="E59" s="144" t="s">
         <v>49</v>
       </c>
-      <c r="F59" s="153"/>
-      <c r="G59" s="154"/>
-      <c r="H59" s="155" t="s">
+      <c r="F59" s="145"/>
+      <c r="G59" s="146"/>
+      <c r="H59" s="147" t="s">
         <v>46</v>
       </c>
-      <c r="I59" s="156"/>
+      <c r="I59" s="148"/>
     </row>
     <row r="60" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A60" s="157" t="s">
+      <c r="A60" s="135" t="s">
         <v>30</v>
       </c>
-      <c r="B60" s="157"/>
+      <c r="B60" s="135"/>
       <c r="C60" s="36"/>
       <c r="D60" s="37"/>
-      <c r="E60" s="158"/>
-      <c r="F60" s="158"/>
-      <c r="G60" s="158"/>
-      <c r="H60" s="159" t="s">
+      <c r="E60" s="136"/>
+      <c r="F60" s="136"/>
+      <c r="G60" s="136"/>
+      <c r="H60" s="137" t="s">
         <v>47</v>
       </c>
-      <c r="I60" s="159"/>
+      <c r="I60" s="137"/>
       <c r="M60" s="38"/>
     </row>
     <row r="61" spans="1:13" ht="13.7" customHeight="1">
-      <c r="A61" s="157" t="s">
+      <c r="A61" s="135" t="s">
         <v>31</v>
       </c>
-      <c r="B61" s="157"/>
+      <c r="B61" s="135"/>
       <c r="C61" s="36"/>
       <c r="D61" s="37"/>
-      <c r="E61" s="158"/>
-      <c r="F61" s="158"/>
-      <c r="G61" s="158"/>
-      <c r="H61" s="159" t="s">
+      <c r="E61" s="136"/>
+      <c r="F61" s="136"/>
+      <c r="G61" s="136"/>
+      <c r="H61" s="137" t="s">
         <v>48</v>
       </c>
-      <c r="I61" s="159"/>
+      <c r="I61" s="137"/>
     </row>
     <row r="62" spans="1:13" ht="13.7" customHeight="1">
       <c r="A62" t="s">
@@ -3543,6 +3673,74 @@
     <row r="17578" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="84">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="B56:I56"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="H57:I57"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="H58:I58"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="E60:G60"/>
+    <mergeCell ref="H60:I60"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="H61:I61"/>
     <mergeCell ref="C51:D51"/>
     <mergeCell ref="C52:D52"/>
     <mergeCell ref="C53:D53"/>
@@ -3559,74 +3757,6 @@
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="C39:D39"/>
     <mergeCell ref="C40:D40"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="E60:G60"/>
-    <mergeCell ref="H60:I60"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="H61:I61"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="E58:G58"/>
-    <mergeCell ref="H58:I58"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="E59:G59"/>
-    <mergeCell ref="H59:I59"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="B55:I55"/>
-    <mergeCell ref="B56:I56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="E57:G57"/>
-    <mergeCell ref="H57:I57"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:I4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:I6"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:I1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:I2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:I3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>